<commit_message>
fix: align recent draft pick metadata
</commit_message>
<xml_diff>
--- a/frontend/public/data/2026/fpros/fpros_merged_formatted.xlsx
+++ b/frontend/public/data/2026/fpros/fpros_merged_formatted.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G303"/>
+  <dimension ref="A1:G307"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -668,7 +668,7 @@
         <v>5</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D6" s="3" t="n">
         <v>8</v>
@@ -761,7 +761,7 @@
         <v>8</v>
       </c>
       <c r="C9" s="5" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D9" s="3" t="n">
         <v>6</v>
@@ -795,7 +795,7 @@
         <v>12</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
@@ -888,7 +888,7 @@
         <v>23</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
@@ -919,7 +919,7 @@
         <v>22</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
@@ -947,7 +947,7 @@
         <v>14</v>
       </c>
       <c r="C15" s="5" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D15" s="3" t="n">
         <v>17</v>
@@ -981,7 +981,7 @@
         <v>21</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
@@ -1008,11 +1008,11 @@
       <c r="B17" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="C17" s="9" t="n">
-        <v>41</v>
+      <c r="C17" s="4" t="n">
+        <v>28</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
@@ -1043,7 +1043,7 @@
         <v>11</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
@@ -1101,11 +1101,11 @@
       <c r="B20" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="C20" s="9" t="n">
-        <v>42</v>
+      <c r="C20" s="4" t="n">
+        <v>26</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
@@ -1136,7 +1136,7 @@
         <v>13</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
@@ -1167,7 +1167,7 @@
         <v>18</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
@@ -1195,10 +1195,10 @@
         <v>22</v>
       </c>
       <c r="C23" s="9" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
@@ -1226,7 +1226,7 @@
         <v>23</v>
       </c>
       <c r="C24" s="9" t="n">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="D24" s="3" t="n">
         <v>27</v>
@@ -1257,10 +1257,10 @@
         <v>24</v>
       </c>
       <c r="C25" s="5" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D25" s="3" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
@@ -1291,7 +1291,7 @@
         <v>29</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
@@ -1322,7 +1322,7 @@
         <v>15</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
@@ -1349,11 +1349,11 @@
       <c r="B28" s="3" t="n">
         <v>27</v>
       </c>
-      <c r="C28" s="4" t="n">
-        <v>33</v>
+      <c r="C28" s="5" t="n">
+        <v>27</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
@@ -1381,10 +1381,10 @@
         <v>28</v>
       </c>
       <c r="C29" s="4" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
@@ -1443,10 +1443,10 @@
         <v>30</v>
       </c>
       <c r="C31" s="5" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="D31" s="3" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
@@ -1474,10 +1474,10 @@
         <v>31</v>
       </c>
       <c r="C32" s="5" t="n">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D32" s="3" t="n">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
@@ -1505,7 +1505,7 @@
         <v>32</v>
       </c>
       <c r="C33" s="9" t="n">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D33" s="3" t="n">
         <v>51</v>
@@ -1539,7 +1539,7 @@
         <v>65</v>
       </c>
       <c r="D34" s="3" t="n">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
@@ -1567,10 +1567,10 @@
         <v>34</v>
       </c>
       <c r="C35" s="5" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D35" s="3" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
@@ -1598,10 +1598,10 @@
         <v>35</v>
       </c>
       <c r="C36" s="7" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D36" s="3" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
@@ -1632,7 +1632,7 @@
         <v>19</v>
       </c>
       <c r="D37" s="3" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
@@ -1659,11 +1659,11 @@
       <c r="B38" s="3" t="n">
         <v>37</v>
       </c>
-      <c r="C38" s="7" t="n">
-        <v>27</v>
+      <c r="C38" s="11" t="n">
+        <v>32</v>
       </c>
       <c r="D38" s="3" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
@@ -1691,7 +1691,7 @@
         <v>38</v>
       </c>
       <c r="C39" s="5" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D39" s="3" t="n">
         <v>35</v>
@@ -1722,10 +1722,10 @@
         <v>39</v>
       </c>
       <c r="C40" s="7" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D40" s="3" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
@@ -1753,10 +1753,10 @@
         <v>40</v>
       </c>
       <c r="C41" s="5" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D41" s="3" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
@@ -1783,11 +1783,11 @@
       <c r="B42" s="3" t="n">
         <v>41</v>
       </c>
-      <c r="C42" s="7" t="n">
-        <v>26</v>
+      <c r="C42" s="5" t="n">
+        <v>38</v>
       </c>
       <c r="D42" s="3" t="n">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
@@ -1818,7 +1818,7 @@
         <v>43</v>
       </c>
       <c r="D43" s="3" t="n">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
@@ -1845,11 +1845,11 @@
       <c r="B44" s="3" t="n">
         <v>43</v>
       </c>
-      <c r="C44" s="9" t="n">
-        <v>57</v>
+      <c r="C44" s="4" t="n">
+        <v>53</v>
       </c>
       <c r="D44" s="3" t="n">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
@@ -1877,10 +1877,10 @@
         <v>44</v>
       </c>
       <c r="C45" s="9" t="n">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="D45" s="3" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
@@ -1907,8 +1907,8 @@
       <c r="B46" s="3" t="n">
         <v>45</v>
       </c>
-      <c r="C46" s="7" t="n">
-        <v>40</v>
+      <c r="C46" s="5" t="n">
+        <v>42</v>
       </c>
       <c r="D46" s="3" t="n">
         <v>33</v>
@@ -1942,7 +1942,7 @@
         <v>49</v>
       </c>
       <c r="D47" s="3" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
@@ -1970,10 +1970,10 @@
         <v>47</v>
       </c>
       <c r="C48" s="7" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D48" s="3" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
@@ -2001,10 +2001,10 @@
         <v>48</v>
       </c>
       <c r="C49" s="7" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D49" s="3" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
@@ -2031,11 +2031,11 @@
       <c r="B50" s="3" t="n">
         <v>49</v>
       </c>
-      <c r="C50" s="5" t="n">
-        <v>51</v>
+      <c r="C50" s="4" t="n">
+        <v>57</v>
       </c>
       <c r="D50" s="3" t="n">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
@@ -2066,7 +2066,7 @@
         <v>48</v>
       </c>
       <c r="D51" s="3" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
@@ -2094,10 +2094,10 @@
         <v>51</v>
       </c>
       <c r="C52" s="5" t="n">
+        <v>51</v>
+      </c>
+      <c r="D52" s="3" t="n">
         <v>50</v>
-      </c>
-      <c r="D52" s="3" t="n">
-        <v>49</v>
       </c>
       <c r="E52" s="3" t="inlineStr">
         <is>
@@ -2125,10 +2125,10 @@
         <v>52</v>
       </c>
       <c r="C53" s="5" t="n">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="D53" s="3" t="n">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
@@ -2155,11 +2155,11 @@
       <c r="B54" s="3" t="n">
         <v>53</v>
       </c>
-      <c r="C54" s="4" t="n">
-        <v>59</v>
+      <c r="C54" s="5" t="n">
+        <v>54</v>
       </c>
       <c r="D54" s="3" t="n">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E54" s="3" t="inlineStr">
         <is>
@@ -2187,10 +2187,10 @@
         <v>54</v>
       </c>
       <c r="C55" s="7" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D55" s="3" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
@@ -2221,7 +2221,7 @@
         <v>66</v>
       </c>
       <c r="D56" s="3" t="n">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E56" s="3" t="inlineStr">
         <is>
@@ -2249,10 +2249,10 @@
         <v>56</v>
       </c>
       <c r="C57" s="5" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="D57" s="3" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
@@ -2280,10 +2280,10 @@
         <v>57</v>
       </c>
       <c r="C58" s="5" t="n">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="D58" s="3" t="n">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
@@ -2311,10 +2311,10 @@
         <v>58</v>
       </c>
       <c r="C59" s="5" t="n">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="D59" s="3" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
@@ -2342,7 +2342,7 @@
         <v>59</v>
       </c>
       <c r="C60" s="5" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D60" s="3" t="n">
         <v>46</v>
@@ -2373,7 +2373,7 @@
         <v>60</v>
       </c>
       <c r="C61" s="5" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D61" s="3" t="n">
         <v>70</v>
@@ -2403,8 +2403,8 @@
       <c r="B62" s="3" t="n">
         <v>61</v>
       </c>
-      <c r="C62" s="7" t="n">
-        <v>54</v>
+      <c r="C62" s="11" t="n">
+        <v>56</v>
       </c>
       <c r="D62" s="3" t="n">
         <v>52</v>
@@ -2435,10 +2435,10 @@
         <v>62</v>
       </c>
       <c r="C63" s="7" t="n">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="D63" s="3" t="n">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
@@ -2466,10 +2466,10 @@
         <v>63</v>
       </c>
       <c r="C64" s="9" t="n">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="D64" s="3" t="n">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
@@ -2497,10 +2497,10 @@
         <v>64</v>
       </c>
       <c r="C65" s="7" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D65" s="3" t="n">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="E65" s="3" t="inlineStr">
         <is>
@@ -2528,7 +2528,7 @@
         <v>65</v>
       </c>
       <c r="C66" s="5" t="n">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D66" s="3" t="n">
         <v>67</v>
@@ -2562,7 +2562,7 @@
         <v>75</v>
       </c>
       <c r="D67" s="3" t="n">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
@@ -2590,10 +2590,10 @@
         <v>67</v>
       </c>
       <c r="C68" s="9" t="n">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D68" s="3" t="n">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="E68" s="3" t="inlineStr">
         <is>
@@ -2621,10 +2621,10 @@
         <v>68</v>
       </c>
       <c r="C69" s="5" t="n">
-        <v>81</v>
+        <v>70</v>
       </c>
       <c r="D69" s="3" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
@@ -2682,11 +2682,11 @@
       <c r="B71" s="3" t="n">
         <v>70</v>
       </c>
-      <c r="C71" s="11" t="n">
-        <v>63</v>
+      <c r="C71" s="7" t="n">
+        <v>61</v>
       </c>
       <c r="D71" s="3" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E71" s="3" t="inlineStr">
         <is>
@@ -2714,10 +2714,10 @@
         <v>71</v>
       </c>
       <c r="C72" s="5" t="n">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="D72" s="3" t="n">
-        <v>75</v>
+        <v>92</v>
       </c>
       <c r="E72" s="3" t="inlineStr">
         <is>
@@ -2745,10 +2745,10 @@
         <v>72</v>
       </c>
       <c r="C73" s="9" t="n">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="D73" s="3" t="n">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="E73" s="3" t="inlineStr">
         <is>
@@ -2775,11 +2775,11 @@
       <c r="B74" s="3" t="n">
         <v>73</v>
       </c>
-      <c r="C74" s="4" t="n">
+      <c r="C74" s="5" t="n">
+        <v>76</v>
+      </c>
+      <c r="D74" s="3" t="n">
         <v>78</v>
-      </c>
-      <c r="D74" s="3" t="n">
-        <v>81</v>
       </c>
       <c r="E74" s="3" t="inlineStr">
         <is>
@@ -2806,11 +2806,11 @@
       <c r="B75" s="3" t="n">
         <v>74</v>
       </c>
-      <c r="C75" s="9" t="n">
-        <v>95</v>
+      <c r="C75" s="4" t="n">
+        <v>86</v>
       </c>
       <c r="D75" s="3" t="n">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="E75" s="3" t="inlineStr">
         <is>
@@ -2838,10 +2838,10 @@
         <v>75</v>
       </c>
       <c r="C76" s="7" t="n">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="D76" s="3" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E76" s="3" t="inlineStr">
         <is>
@@ -2869,10 +2869,10 @@
         <v>76</v>
       </c>
       <c r="C77" s="9" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D77" s="3" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="E77" s="3" t="inlineStr">
         <is>
@@ -2900,7 +2900,7 @@
         <v>77</v>
       </c>
       <c r="C78" s="5" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D78" s="3" t="n">
         <v>80</v>
@@ -2930,11 +2930,11 @@
       <c r="B79" s="3" t="n">
         <v>78</v>
       </c>
-      <c r="C79" s="11" t="n">
-        <v>72</v>
+      <c r="C79" s="5" t="n">
+        <v>78</v>
       </c>
       <c r="D79" s="3" t="n">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="E79" s="3" t="inlineStr">
         <is>
@@ -2962,7 +2962,7 @@
         <v>79</v>
       </c>
       <c r="C80" s="5" t="n">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D80" s="3" t="n">
         <v>68</v>
@@ -2992,11 +2992,11 @@
       <c r="B81" s="3" t="n">
         <v>80</v>
       </c>
-      <c r="C81" s="4" t="n">
-        <v>85</v>
+      <c r="C81" s="9" t="n">
+        <v>94</v>
       </c>
       <c r="D81" s="3" t="n">
-        <v>109</v>
+        <v>98</v>
       </c>
       <c r="E81" s="3" t="inlineStr">
         <is>
@@ -3024,7 +3024,7 @@
         <v>81</v>
       </c>
       <c r="C82" s="7" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D82" s="3" t="n">
         <v>69</v>
@@ -3054,11 +3054,11 @@
       <c r="B83" s="3" t="n">
         <v>82</v>
       </c>
-      <c r="C83" s="9" t="n">
-        <v>127</v>
+      <c r="C83" s="5" t="n">
+        <v>99</v>
       </c>
       <c r="D83" s="3" t="n">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="E83" s="3" t="inlineStr">
         <is>
@@ -3086,10 +3086,10 @@
         <v>83</v>
       </c>
       <c r="C84" s="9" t="n">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="D84" s="3" t="n">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E84" s="3" t="inlineStr">
         <is>
@@ -3116,11 +3116,11 @@
       <c r="B85" s="3" t="n">
         <v>84</v>
       </c>
-      <c r="C85" s="7" t="n">
-        <v>74</v>
+      <c r="C85" s="5" t="n">
+        <v>92</v>
       </c>
       <c r="D85" s="3" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E85" s="3" t="inlineStr">
         <is>
@@ -3148,10 +3148,10 @@
         <v>85</v>
       </c>
       <c r="C86" s="5" t="n">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="D86" s="3" t="n">
-        <v>104</v>
+        <v>116</v>
       </c>
       <c r="E86" s="3" t="inlineStr">
         <is>
@@ -3178,11 +3178,11 @@
       <c r="B87" s="3" t="n">
         <v>86</v>
       </c>
-      <c r="C87" s="5" t="n">
-        <v>77</v>
+      <c r="C87" s="9" t="n">
+        <v>107</v>
       </c>
       <c r="D87" s="3" t="n">
-        <v>92</v>
+        <v>129</v>
       </c>
       <c r="E87" s="3" t="inlineStr">
         <is>
@@ -3210,10 +3210,10 @@
         <v>87</v>
       </c>
       <c r="C88" s="9" t="n">
-        <v>149</v>
+        <v>139</v>
       </c>
       <c r="D88" s="3" t="n">
-        <v>143</v>
+        <v>163</v>
       </c>
       <c r="E88" s="3" t="inlineStr">
         <is>
@@ -3241,10 +3241,10 @@
         <v>88</v>
       </c>
       <c r="C89" s="7" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D89" s="3" t="n">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E89" s="3" t="inlineStr">
         <is>
@@ -3272,10 +3272,10 @@
         <v>89</v>
       </c>
       <c r="C90" s="5" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D90" s="3" t="n">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="E90" s="3" t="inlineStr">
         <is>
@@ -3303,10 +3303,10 @@
         <v>90</v>
       </c>
       <c r="C91" s="5" t="n">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D91" s="3" t="n">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="E91" s="3" t="inlineStr">
         <is>
@@ -3334,10 +3334,10 @@
         <v>91</v>
       </c>
       <c r="C92" s="9" t="n">
-        <v>112</v>
+        <v>122</v>
       </c>
       <c r="D92" s="3" t="n">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="E92" s="3" t="inlineStr">
         <is>
@@ -3365,7 +3365,7 @@
         <v>92</v>
       </c>
       <c r="C93" s="7" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D93" s="3" t="n">
         <v>47</v>
@@ -3396,10 +3396,10 @@
         <v>93</v>
       </c>
       <c r="C94" s="9" t="n">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="D94" s="3" t="n">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="E94" s="3" t="inlineStr">
         <is>
@@ -3427,10 +3427,10 @@
         <v>94</v>
       </c>
       <c r="C95" s="9" t="n">
-        <v>113</v>
+        <v>124</v>
       </c>
       <c r="D95" s="3" t="n">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="E95" s="3" t="inlineStr">
         <is>
@@ -3458,10 +3458,10 @@
         <v>95</v>
       </c>
       <c r="C96" s="5" t="n">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="D96" s="3" t="n">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="E96" s="3" t="inlineStr">
         <is>
@@ -3489,10 +3489,10 @@
         <v>96</v>
       </c>
       <c r="C97" s="5" t="n">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="D97" s="3" t="n">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E97" s="3" t="inlineStr">
         <is>
@@ -3520,10 +3520,10 @@
         <v>97</v>
       </c>
       <c r="C98" s="5" t="n">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="D98" s="3" t="n">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="E98" s="3" t="inlineStr">
         <is>
@@ -3551,10 +3551,10 @@
         <v>98</v>
       </c>
       <c r="C99" s="5" t="n">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="D99" s="3" t="n">
-        <v>94</v>
+        <v>115</v>
       </c>
       <c r="E99" s="3" t="inlineStr">
         <is>
@@ -3582,10 +3582,10 @@
         <v>99</v>
       </c>
       <c r="C100" s="9" t="n">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D100" s="3" t="n">
-        <v>129</v>
+        <v>138</v>
       </c>
       <c r="E100" s="3" t="inlineStr">
         <is>
@@ -3613,10 +3613,10 @@
         <v>101</v>
       </c>
       <c r="C101" s="5" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D101" s="3" t="n">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E101" s="3" t="inlineStr">
         <is>
@@ -3644,10 +3644,10 @@
         <v>102</v>
       </c>
       <c r="C102" s="5" t="n">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="D102" s="3" t="n">
-        <v>144</v>
+        <v>131</v>
       </c>
       <c r="E102" s="3" t="inlineStr">
         <is>
@@ -3675,10 +3675,10 @@
         <v>103</v>
       </c>
       <c r="C103" s="5" t="n">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D103" s="3" t="n">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E103" s="3" t="inlineStr">
         <is>
@@ -3706,10 +3706,10 @@
         <v>104</v>
       </c>
       <c r="C104" s="5" t="n">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D104" s="3" t="n">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="E104" s="3" t="inlineStr">
         <is>
@@ -3737,7 +3737,7 @@
         <v>105</v>
       </c>
       <c r="C105" s="5" t="n">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="D105" s="3" t="n">
         <v>154</v>
@@ -3768,10 +3768,10 @@
         <v>106</v>
       </c>
       <c r="C106" s="5" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D106" s="3" t="n">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="E106" s="3" t="inlineStr">
         <is>
@@ -3799,10 +3799,10 @@
         <v>107</v>
       </c>
       <c r="C107" s="7" t="n">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D107" s="3" t="n">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="E107" s="3" t="inlineStr">
         <is>
@@ -3830,10 +3830,10 @@
         <v>108</v>
       </c>
       <c r="C108" s="5" t="n">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="D108" s="3" t="n">
-        <v>145</v>
+        <v>132</v>
       </c>
       <c r="E108" s="3" t="inlineStr">
         <is>
@@ -3860,11 +3860,11 @@
       <c r="B109" s="3" t="n">
         <v>109</v>
       </c>
-      <c r="C109" s="5" t="n">
-        <v>114</v>
+      <c r="C109" s="9" t="n">
+        <v>123</v>
       </c>
       <c r="D109" s="3" t="n">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="E109" s="3" t="inlineStr">
         <is>
@@ -3891,11 +3891,11 @@
       <c r="B110" s="3" t="n">
         <v>110</v>
       </c>
-      <c r="C110" s="7" t="n">
-        <v>98</v>
+      <c r="C110" s="11" t="n">
+        <v>104</v>
       </c>
       <c r="D110" s="3" t="n">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="E110" s="3" t="inlineStr">
         <is>
@@ -3922,11 +3922,11 @@
       <c r="B111" s="3" t="n">
         <v>111</v>
       </c>
-      <c r="C111" s="5" t="n">
-        <v>125</v>
+      <c r="C111" s="7" t="n">
+        <v>97</v>
       </c>
       <c r="D111" s="3" t="n">
-        <v>116</v>
+        <v>104</v>
       </c>
       <c r="E111" s="3" t="inlineStr">
         <is>
@@ -3957,7 +3957,7 @@
         <v>93</v>
       </c>
       <c r="D112" s="3" t="n">
-        <v>111</v>
+        <v>97</v>
       </c>
       <c r="E112" s="3" t="inlineStr">
         <is>
@@ -3985,10 +3985,10 @@
         <v>113</v>
       </c>
       <c r="C113" s="7" t="n">
-        <v>90</v>
+        <v>102</v>
       </c>
       <c r="D113" s="3" t="n">
-        <v>102</v>
+        <v>112</v>
       </c>
       <c r="E113" s="3" t="inlineStr">
         <is>
@@ -4016,10 +4016,10 @@
         <v>114</v>
       </c>
       <c r="C114" s="5" t="n">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D114" s="3" t="n">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="E114" s="3" t="inlineStr">
         <is>
@@ -4046,11 +4046,11 @@
       <c r="B115" s="3" t="n">
         <v>115</v>
       </c>
-      <c r="C115" s="11" t="n">
-        <v>108</v>
+      <c r="C115" s="7" t="n">
+        <v>96</v>
       </c>
       <c r="D115" s="3" t="n">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="E115" s="3" t="inlineStr">
         <is>
@@ -4077,11 +4077,11 @@
       <c r="B116" s="3" t="n">
         <v>116</v>
       </c>
-      <c r="C116" s="4" t="n">
-        <v>124</v>
+      <c r="C116" s="9" t="n">
+        <v>137</v>
       </c>
       <c r="D116" s="3" t="n">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="E116" s="3" t="inlineStr">
         <is>
@@ -4109,10 +4109,10 @@
         <v>117</v>
       </c>
       <c r="C117" s="5" t="n">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="D117" s="3" t="n">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="E117" s="3" t="inlineStr">
         <is>
@@ -4140,10 +4140,10 @@
         <v>118</v>
       </c>
       <c r="C118" s="5" t="n">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D118" s="3" t="n">
-        <v>130</v>
+        <v>139</v>
       </c>
       <c r="E118" s="3" t="inlineStr">
         <is>
@@ -4170,11 +4170,11 @@
       <c r="B119" s="3" t="n">
         <v>119</v>
       </c>
-      <c r="C119" s="5" t="n">
-        <v>119</v>
+      <c r="C119" s="11" t="n">
+        <v>113</v>
       </c>
       <c r="D119" s="3" t="n">
-        <v>133</v>
+        <v>123</v>
       </c>
       <c r="E119" s="3" t="inlineStr">
         <is>
@@ -4202,10 +4202,10 @@
         <v>120</v>
       </c>
       <c r="C120" s="5" t="n">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="D120" s="3" t="n">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E120" s="3" t="inlineStr">
         <is>
@@ -4233,10 +4233,10 @@
         <v>121</v>
       </c>
       <c r="C121" s="5" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D121" s="3" t="n">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="E121" s="3" t="inlineStr">
         <is>
@@ -4264,10 +4264,10 @@
         <v>122</v>
       </c>
       <c r="C122" s="9" t="n">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="D122" s="3" t="n">
-        <v>174</v>
+        <v>185</v>
       </c>
       <c r="E122" s="3" t="inlineStr">
         <is>
@@ -4295,10 +4295,10 @@
         <v>123</v>
       </c>
       <c r="C123" s="7" t="n">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="D123" s="3" t="n">
-        <v>117</v>
+        <v>105</v>
       </c>
       <c r="E123" s="3" t="inlineStr">
         <is>
@@ -4326,10 +4326,10 @@
         <v>124</v>
       </c>
       <c r="C124" s="7" t="n">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D124" s="3" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E124" s="3" t="inlineStr">
         <is>
@@ -4356,11 +4356,11 @@
       <c r="B125" s="3" t="n">
         <v>125</v>
       </c>
-      <c r="C125" s="7" t="n">
-        <v>102</v>
+      <c r="C125" s="5" t="n">
+        <v>126</v>
       </c>
       <c r="D125" s="3" t="n">
-        <v>103</v>
+        <v>113</v>
       </c>
       <c r="E125" s="3" t="inlineStr">
         <is>
@@ -4387,11 +4387,11 @@
       <c r="B126" s="3" t="n">
         <v>126</v>
       </c>
-      <c r="C126" s="4" t="n">
-        <v>135</v>
+      <c r="C126" s="7" t="n">
+        <v>82</v>
       </c>
       <c r="D126" s="3" t="n">
-        <v>110</v>
+        <v>87</v>
       </c>
       <c r="E126" s="3" t="inlineStr">
         <is>
@@ -4422,7 +4422,7 @@
         <v>120</v>
       </c>
       <c r="D127" s="3" t="n">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="E127" s="3" t="inlineStr">
         <is>
@@ -4450,7 +4450,7 @@
         <v>128</v>
       </c>
       <c r="C128" s="7" t="n">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="D128" s="3" t="n">
         <v>76</v>
@@ -4480,11 +4480,11 @@
       <c r="B129" s="3" t="n">
         <v>129</v>
       </c>
-      <c r="C129" s="7" t="n">
-        <v>117</v>
+      <c r="C129" s="9" t="n">
+        <v>201</v>
       </c>
       <c r="D129" s="3" t="n">
-        <v>171</v>
+        <v>197</v>
       </c>
       <c r="E129" s="3" t="inlineStr">
         <is>
@@ -4512,10 +4512,10 @@
         <v>130</v>
       </c>
       <c r="C130" s="5" t="n">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="D130" s="3" t="n">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="E130" s="3" t="inlineStr">
         <is>
@@ -4543,10 +4543,10 @@
         <v>131</v>
       </c>
       <c r="C131" s="9" t="n">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D131" s="3" t="n">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="E131" s="3" t="inlineStr">
         <is>
@@ -4573,11 +4573,11 @@
       <c r="B132" s="3" t="n">
         <v>132</v>
       </c>
-      <c r="C132" s="5" t="n">
-        <v>136</v>
+      <c r="C132" s="4" t="n">
+        <v>141</v>
       </c>
       <c r="D132" s="3" t="n">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E132" s="3" t="inlineStr">
         <is>
@@ -4605,10 +4605,10 @@
         <v>133</v>
       </c>
       <c r="C133" s="7" t="n">
-        <v>58</v>
+        <v>73</v>
       </c>
       <c r="D133" s="3" t="n">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E133" s="3" t="inlineStr">
         <is>
@@ -4636,10 +4636,10 @@
         <v>134</v>
       </c>
       <c r="C134" s="9" t="n">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="D134" s="3" t="n">
-        <v>173</v>
+        <v>184</v>
       </c>
       <c r="E134" s="3" t="inlineStr">
         <is>
@@ -4667,10 +4667,10 @@
         <v>135</v>
       </c>
       <c r="C135" s="5" t="n">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D135" s="3" t="n">
-        <v>152</v>
+        <v>141</v>
       </c>
       <c r="E135" s="3" t="inlineStr">
         <is>
@@ -4698,10 +4698,10 @@
         <v>136</v>
       </c>
       <c r="C136" s="5" t="n">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="D136" s="3" t="n">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="E136" s="3" t="inlineStr">
         <is>
@@ -4729,10 +4729,10 @@
         <v>137</v>
       </c>
       <c r="C137" s="5" t="n">
-        <v>176</v>
+        <v>147</v>
       </c>
       <c r="D137" s="3" t="n">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="E137" s="3" t="inlineStr">
         <is>
@@ -4760,10 +4760,10 @@
         <v>138</v>
       </c>
       <c r="C138" s="9" t="n">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="D138" s="3" t="n">
-        <v>175</v>
+        <v>186</v>
       </c>
       <c r="E138" s="3" t="inlineStr">
         <is>
@@ -4790,11 +4790,11 @@
       <c r="B139" s="3" t="n">
         <v>139</v>
       </c>
-      <c r="C139" s="5" t="n">
-        <v>161</v>
+      <c r="C139" s="7" t="n">
+        <v>125</v>
       </c>
       <c r="D139" s="3" t="n">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="E139" s="3" t="inlineStr">
         <is>
@@ -4821,11 +4821,11 @@
       <c r="B140" s="3" t="n">
         <v>140</v>
       </c>
-      <c r="C140" s="7" t="n">
-        <v>128</v>
+      <c r="C140" s="5" t="n">
+        <v>148</v>
       </c>
       <c r="D140" s="3" t="n">
-        <v>151</v>
+        <v>142</v>
       </c>
       <c r="E140" s="3" t="inlineStr">
         <is>
@@ -4853,10 +4853,10 @@
         <v>141</v>
       </c>
       <c r="C141" s="5" t="n">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="D141" s="3" t="n">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="E141" s="3" t="inlineStr">
         <is>
@@ -4884,10 +4884,10 @@
         <v>142</v>
       </c>
       <c r="C142" s="5" t="n">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D142" s="3" t="n">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="E142" s="3" t="inlineStr">
         <is>
@@ -4915,10 +4915,10 @@
         <v>143</v>
       </c>
       <c r="C143" s="5" t="n">
-        <v>204</v>
+        <v>211</v>
       </c>
       <c r="D143" s="3" t="n">
-        <v>214</v>
+        <v>227</v>
       </c>
       <c r="E143" s="3" t="inlineStr">
         <is>
@@ -4946,10 +4946,10 @@
         <v>144</v>
       </c>
       <c r="C144" s="5" t="n">
-        <v>198</v>
+        <v>210</v>
       </c>
       <c r="D144" s="3" t="n">
-        <v>195</v>
+        <v>202</v>
       </c>
       <c r="E144" s="3" t="inlineStr">
         <is>
@@ -4977,10 +4977,10 @@
         <v>145</v>
       </c>
       <c r="C145" s="9" t="n">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D145" s="3" t="n">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="E145" s="3" t="inlineStr">
         <is>
@@ -5008,10 +5008,10 @@
         <v>146</v>
       </c>
       <c r="C146" s="5" t="n">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="D146" s="3" t="n">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="E146" s="3" t="inlineStr">
         <is>
@@ -5070,10 +5070,10 @@
         <v>148</v>
       </c>
       <c r="C148" s="9" t="n">
-        <v>191</v>
+        <v>223</v>
       </c>
       <c r="D148" s="3" t="n">
-        <v>206</v>
+        <v>217</v>
       </c>
       <c r="E148" s="3" t="inlineStr">
         <is>
@@ -5100,11 +5100,11 @@
       <c r="B149" s="3" t="n">
         <v>149</v>
       </c>
-      <c r="C149" s="11" t="n">
-        <v>106</v>
+      <c r="C149" s="5" t="n">
+        <v>151</v>
       </c>
       <c r="D149" s="3" t="n">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E149" s="3" t="inlineStr">
         <is>
@@ -5132,10 +5132,10 @@
         <v>150</v>
       </c>
       <c r="C150" s="4" t="n">
-        <v>202</v>
+        <v>255</v>
       </c>
       <c r="D150" s="3" t="n">
-        <v>219</v>
+        <v>229</v>
       </c>
       <c r="E150" s="3" t="inlineStr">
         <is>
@@ -5163,10 +5163,10 @@
         <v>151</v>
       </c>
       <c r="C151" s="4" t="n">
-        <v>206</v>
+        <v>217</v>
       </c>
       <c r="D151" s="3" t="n">
-        <v>181</v>
+        <v>194</v>
       </c>
       <c r="E151" s="3" t="inlineStr">
         <is>
@@ -5194,10 +5194,10 @@
         <v>152</v>
       </c>
       <c r="C152" s="4" t="n">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="D152" s="3" t="n">
-        <v>180</v>
+        <v>193</v>
       </c>
       <c r="E152" s="3" t="inlineStr">
         <is>
@@ -5225,10 +5225,10 @@
         <v>153</v>
       </c>
       <c r="C153" s="4" t="n">
-        <v>200</v>
+        <v>222</v>
       </c>
       <c r="D153" s="3" t="n">
-        <v>205</v>
+        <v>216</v>
       </c>
       <c r="E153" s="3" t="inlineStr">
         <is>
@@ -5256,10 +5256,10 @@
         <v>154</v>
       </c>
       <c r="C154" s="5" t="n">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D154" s="3" t="n">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="E154" s="3" t="inlineStr">
         <is>
@@ -5287,10 +5287,10 @@
         <v>155</v>
       </c>
       <c r="C155" s="4" t="n">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="D155" s="3" t="n">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="E155" s="3" t="inlineStr">
         <is>
@@ -5317,11 +5317,11 @@
       <c r="B156" s="3" t="n">
         <v>156</v>
       </c>
-      <c r="C156" s="11" t="n">
-        <v>146</v>
+      <c r="C156" s="5" t="n">
+        <v>174</v>
       </c>
       <c r="D156" s="3" t="n">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="E156" s="3" t="inlineStr">
         <is>
@@ -5349,10 +5349,10 @@
         <v>158</v>
       </c>
       <c r="C157" s="5" t="n">
-        <v>210</v>
+        <v>179</v>
       </c>
       <c r="D157" s="3" t="n">
-        <v>191</v>
+        <v>177</v>
       </c>
       <c r="E157" s="3" t="inlineStr">
         <is>
@@ -5380,10 +5380,10 @@
         <v>159</v>
       </c>
       <c r="C158" s="7" t="n">
-        <v>144</v>
+        <v>101</v>
       </c>
       <c r="D158" s="3" t="n">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="E158" s="3" t="inlineStr">
         <is>
@@ -5414,7 +5414,7 @@
         <v>190</v>
       </c>
       <c r="D159" s="3" t="n">
-        <v>198</v>
+        <v>180</v>
       </c>
       <c r="E159" s="3" t="inlineStr">
         <is>
@@ -5442,10 +5442,10 @@
         <v>161</v>
       </c>
       <c r="C160" s="5" t="n">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D160" s="3" t="n">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E160" s="3" t="inlineStr">
         <is>
@@ -5473,10 +5473,10 @@
         <v>162</v>
       </c>
       <c r="C161" s="4" t="n">
-        <v>235</v>
+        <v>225</v>
       </c>
       <c r="D161" s="3" t="n">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="E161" s="3" t="inlineStr">
         <is>
@@ -5504,10 +5504,10 @@
         <v>164</v>
       </c>
       <c r="C162" s="4" t="n">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="D162" s="3" t="n">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="E162" s="3" t="inlineStr">
         <is>
@@ -5535,10 +5535,10 @@
         <v>165</v>
       </c>
       <c r="C163" s="5" t="n">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D163" s="3" t="n">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="E163" s="3" t="inlineStr">
         <is>
@@ -5566,10 +5566,10 @@
         <v>166</v>
       </c>
       <c r="C164" s="4" t="n">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="D164" s="3" t="n">
-        <v>224</v>
+        <v>211</v>
       </c>
       <c r="E164" s="3" t="inlineStr">
         <is>
@@ -5597,10 +5597,10 @@
         <v>167</v>
       </c>
       <c r="C165" s="5" t="n">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D165" s="3" t="n">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="E165" s="3" t="inlineStr">
         <is>
@@ -5627,11 +5627,11 @@
       <c r="B166" s="3" t="n">
         <v>169</v>
       </c>
-      <c r="C166" s="4" t="n">
-        <v>269</v>
+      <c r="C166" s="5" t="n">
+        <v>177</v>
       </c>
       <c r="D166" s="3" t="n">
-        <v>196</v>
+        <v>176</v>
       </c>
       <c r="E166" s="3" t="inlineStr">
         <is>
@@ -5659,10 +5659,10 @@
         <v>170</v>
       </c>
       <c r="C167" s="5" t="n">
-        <v>189</v>
+        <v>172</v>
       </c>
       <c r="D167" s="3" t="n">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="E167" s="3" t="inlineStr">
         <is>
@@ -5690,10 +5690,10 @@
         <v>173</v>
       </c>
       <c r="C168" s="5" t="n">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D168" s="3" t="n">
-        <v>222</v>
+        <v>205</v>
       </c>
       <c r="E168" s="3" t="inlineStr">
         <is>
@@ -5721,10 +5721,10 @@
         <v>174</v>
       </c>
       <c r="C169" s="4" t="n">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="D169" s="3" t="n">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="E169" s="3" t="inlineStr">
         <is>
@@ -5752,10 +5752,10 @@
         <v>175</v>
       </c>
       <c r="C170" s="4" t="n">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="D170" s="3" t="n">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="E170" s="3" t="inlineStr">
         <is>
@@ -5786,7 +5786,7 @@
         <v>171</v>
       </c>
       <c r="D171" s="3" t="n">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="E171" s="3" t="inlineStr">
         <is>
@@ -5814,10 +5814,10 @@
         <v>177</v>
       </c>
       <c r="C172" s="7" t="n">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="D172" s="3" t="n">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="E172" s="3" t="inlineStr">
         <is>
@@ -5845,10 +5845,10 @@
         <v>178</v>
       </c>
       <c r="C173" s="4" t="n">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D173" s="3" t="n">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="E173" s="3" t="inlineStr">
         <is>
@@ -5879,7 +5879,7 @@
         <v>237</v>
       </c>
       <c r="D174" s="3" t="n">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="E174" s="3" t="inlineStr">
         <is>
@@ -5907,10 +5907,10 @@
         <v>185</v>
       </c>
       <c r="C175" s="4" t="n">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="D175" s="3" t="n">
-        <v>277</v>
+        <v>268</v>
       </c>
       <c r="E175" s="3" t="inlineStr">
         <is>
@@ -5938,10 +5938,10 @@
         <v>186</v>
       </c>
       <c r="C176" s="4" t="n">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="D176" s="3" t="n">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="E176" s="3" t="inlineStr">
         <is>
@@ -5969,10 +5969,10 @@
         <v>187</v>
       </c>
       <c r="C177" s="4" t="n">
-        <v>225</v>
+        <v>254</v>
       </c>
       <c r="D177" s="3" t="n">
-        <v>221</v>
+        <v>231</v>
       </c>
       <c r="E177" s="3" t="inlineStr">
         <is>
@@ -6000,10 +6000,10 @@
         <v>188</v>
       </c>
       <c r="C178" s="4" t="n">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="D178" s="3" t="n">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="E178" s="3" t="inlineStr">
         <is>
@@ -6034,7 +6034,7 @@
         <v>279</v>
       </c>
       <c r="D179" s="3" t="n">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="E179" s="3" t="inlineStr">
         <is>
@@ -6061,11 +6061,11 @@
       <c r="B180" s="3" t="n">
         <v>192</v>
       </c>
-      <c r="C180" s="4" t="n">
-        <v>273</v>
+      <c r="C180" s="5" t="n">
+        <v>195</v>
       </c>
       <c r="D180" s="3" t="n">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="E180" s="3" t="inlineStr">
         <is>
@@ -6093,10 +6093,10 @@
         <v>194</v>
       </c>
       <c r="C181" s="4" t="n">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D181" s="3" t="n">
-        <v>256</v>
+        <v>271</v>
       </c>
       <c r="E181" s="3" t="inlineStr">
         <is>
@@ -6123,11 +6123,11 @@
       <c r="B182" s="3" t="n">
         <v>195</v>
       </c>
-      <c r="C182" s="11" t="n">
-        <v>163</v>
+      <c r="C182" s="5" t="n">
+        <v>176</v>
       </c>
       <c r="D182" s="3" t="n">
-        <v>188</v>
+        <v>168</v>
       </c>
       <c r="E182" s="3" t="inlineStr">
         <is>
@@ -6154,11 +6154,11 @@
       <c r="B183" s="3" t="n">
         <v>196</v>
       </c>
-      <c r="C183" s="5" t="n">
-        <v>174</v>
+      <c r="C183" s="11" t="n">
+        <v>159</v>
       </c>
       <c r="D183" s="3" t="n">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="E183" s="3" t="inlineStr">
         <is>
@@ -6186,10 +6186,10 @@
         <v>197</v>
       </c>
       <c r="C184" s="4" t="n">
-        <v>294</v>
+        <v>300</v>
       </c>
       <c r="D184" s="3" t="n">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="E184" s="3" t="inlineStr">
         <is>
@@ -6216,11 +6216,11 @@
       <c r="B185" s="3" t="n">
         <v>199</v>
       </c>
-      <c r="C185" s="5" t="n">
-        <v>170</v>
+      <c r="C185" s="11" t="n">
+        <v>161</v>
       </c>
       <c r="D185" s="3" t="n">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="E185" s="3" t="inlineStr">
         <is>
@@ -6248,10 +6248,10 @@
         <v>201</v>
       </c>
       <c r="C186" s="11" t="n">
-        <v>158</v>
+        <v>170</v>
       </c>
       <c r="D186" s="3" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="E186" s="3" t="inlineStr">
         <is>
@@ -6279,10 +6279,10 @@
         <v>202</v>
       </c>
       <c r="C187" s="5" t="n">
-        <v>172</v>
+        <v>202</v>
       </c>
       <c r="D187" s="3" t="n">
-        <v>197</v>
+        <v>230</v>
       </c>
       <c r="E187" s="3" t="inlineStr">
         <is>
@@ -6310,10 +6310,10 @@
         <v>204</v>
       </c>
       <c r="C188" s="11" t="n">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D188" s="3" t="n">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E188" s="3" t="inlineStr">
         <is>
@@ -6341,10 +6341,10 @@
         <v>205</v>
       </c>
       <c r="C189" s="5" t="n">
-        <v>222</v>
+        <v>205</v>
       </c>
       <c r="D189" s="3" t="n">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="E189" s="3" t="inlineStr">
         <is>
@@ -6372,10 +6372,10 @@
         <v>206</v>
       </c>
       <c r="C190" s="4" t="n">
-        <v>268</v>
+        <v>295</v>
       </c>
       <c r="D190" s="3" t="n">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="E190" s="3" t="inlineStr">
         <is>
@@ -6403,10 +6403,10 @@
         <v>207</v>
       </c>
       <c r="C191" s="4" t="n">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="D191" s="3" t="n">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="E191" s="3" t="inlineStr">
         <is>
@@ -6437,7 +6437,7 @@
         <v>173</v>
       </c>
       <c r="D192" s="3" t="n">
-        <v>183</v>
+        <v>167</v>
       </c>
       <c r="E192" s="3" t="inlineStr">
         <is>
@@ -6465,10 +6465,10 @@
         <v>212</v>
       </c>
       <c r="C193" s="5" t="n">
-        <v>211</v>
+        <v>240</v>
       </c>
       <c r="D193" s="3" t="n">
-        <v>215</v>
+        <v>228</v>
       </c>
       <c r="E193" s="3" t="inlineStr">
         <is>
@@ -6496,10 +6496,10 @@
         <v>213</v>
       </c>
       <c r="C194" s="4" t="n">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="D194" s="3" t="n">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="E194" s="3" t="inlineStr">
         <is>
@@ -6527,10 +6527,10 @@
         <v>217</v>
       </c>
       <c r="C195" s="4" t="n">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="D195" s="3" t="n">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="E195" s="3" t="inlineStr">
         <is>
@@ -6558,10 +6558,10 @@
         <v>219</v>
       </c>
       <c r="C196" s="5" t="n">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="D196" s="3" t="n">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="E196" s="3" t="inlineStr">
         <is>
@@ -6589,10 +6589,10 @@
         <v>221</v>
       </c>
       <c r="C197" s="4" t="n">
-        <v>265</v>
+        <v>283</v>
       </c>
       <c r="D197" s="3" t="n">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="E197" s="3" t="inlineStr">
         <is>
@@ -6619,11 +6619,11 @@
       <c r="B198" s="3" t="n">
         <v>222</v>
       </c>
-      <c r="C198" s="5" t="n">
-        <v>240</v>
+      <c r="C198" s="4" t="n">
+        <v>269</v>
       </c>
       <c r="D198" s="3" t="n">
-        <v>245</v>
+        <v>239</v>
       </c>
       <c r="E198" s="3" t="inlineStr">
         <is>
@@ -6654,7 +6654,7 @@
         <v>218</v>
       </c>
       <c r="D199" s="3" t="n">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="E199" s="3" t="inlineStr">
         <is>
@@ -6682,7 +6682,7 @@
         <v>224</v>
       </c>
       <c r="C200" s="4" t="n">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="D200" s="3" t="inlineStr"/>
       <c r="E200" s="3" t="inlineStr">
@@ -6711,10 +6711,10 @@
         <v>225</v>
       </c>
       <c r="C201" s="7" t="n">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="D201" s="3" t="n">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E201" s="3" t="inlineStr">
         <is>
@@ -6741,11 +6741,11 @@
       <c r="B202" s="3" t="n">
         <v>228</v>
       </c>
-      <c r="C202" s="5" t="n">
-        <v>257</v>
+      <c r="C202" s="4" t="n">
+        <v>263</v>
       </c>
       <c r="D202" s="3" t="n">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="E202" s="3" t="inlineStr">
         <is>
@@ -6772,11 +6772,11 @@
       <c r="B203" s="3" t="n">
         <v>230</v>
       </c>
-      <c r="C203" s="5" t="n">
-        <v>224</v>
+      <c r="C203" s="11" t="n">
+        <v>192</v>
       </c>
       <c r="D203" s="3" t="n">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="E203" s="3" t="inlineStr">
         <is>
@@ -6803,11 +6803,11 @@
       <c r="B204" s="3" t="n">
         <v>232</v>
       </c>
-      <c r="C204" s="5" t="n">
-        <v>266</v>
+      <c r="C204" s="4" t="n">
+        <v>299</v>
       </c>
       <c r="D204" s="3" t="n">
-        <v>253</v>
+        <v>300</v>
       </c>
       <c r="E204" s="3" t="inlineStr">
         <is>
@@ -6835,10 +6835,10 @@
         <v>233</v>
       </c>
       <c r="C205" s="4" t="n">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="D205" s="3" t="n">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="E205" s="3" t="inlineStr">
         <is>
@@ -6866,10 +6866,10 @@
         <v>234</v>
       </c>
       <c r="C206" s="5" t="n">
-        <v>217</v>
+        <v>206</v>
       </c>
       <c r="D206" s="3" t="n">
-        <v>199</v>
+        <v>192</v>
       </c>
       <c r="E206" s="3" t="inlineStr">
         <is>
@@ -6897,10 +6897,10 @@
         <v>235</v>
       </c>
       <c r="C207" s="5" t="n">
-        <v>245</v>
+        <v>259</v>
       </c>
       <c r="D207" s="3" t="n">
-        <v>273</v>
+        <v>260</v>
       </c>
       <c r="E207" s="3" t="inlineStr">
         <is>
@@ -6928,10 +6928,10 @@
         <v>237</v>
       </c>
       <c r="C208" s="5" t="n">
-        <v>256</v>
+        <v>265</v>
       </c>
       <c r="D208" s="3" t="n">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="E208" s="3" t="inlineStr">
         <is>
@@ -6959,10 +6959,10 @@
         <v>238</v>
       </c>
       <c r="C209" s="5" t="n">
-        <v>221</v>
+        <v>234</v>
       </c>
       <c r="D209" s="3" t="n">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="E209" s="3" t="inlineStr">
         <is>
@@ -6989,11 +6989,11 @@
       <c r="B210" s="3" t="n">
         <v>239</v>
       </c>
-      <c r="C210" s="5" t="n">
-        <v>260</v>
+      <c r="C210" s="4" t="n">
+        <v>281</v>
       </c>
       <c r="D210" s="3" t="n">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="E210" s="3" t="inlineStr">
         <is>
@@ -7021,10 +7021,10 @@
         <v>240</v>
       </c>
       <c r="C211" s="5" t="n">
-        <v>238</v>
+        <v>270</v>
       </c>
       <c r="D211" s="3" t="n">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="E211" s="3" t="inlineStr">
         <is>
@@ -7055,7 +7055,7 @@
         <v>291</v>
       </c>
       <c r="D212" s="3" t="n">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="E212" s="3" t="inlineStr">
         <is>
@@ -7082,11 +7082,11 @@
       <c r="B213" s="3" t="n">
         <v>242</v>
       </c>
-      <c r="C213" s="4" t="n">
-        <v>300</v>
+      <c r="C213" s="5" t="n">
+        <v>264</v>
       </c>
       <c r="D213" s="3" t="n">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="E213" s="3" t="inlineStr">
         <is>
@@ -7114,10 +7114,10 @@
         <v>243</v>
       </c>
       <c r="C214" s="5" t="n">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="D214" s="3" t="n">
-        <v>226</v>
+        <v>213</v>
       </c>
       <c r="E214" s="3" t="inlineStr">
         <is>
@@ -7145,10 +7145,10 @@
         <v>244</v>
       </c>
       <c r="C215" s="4" t="n">
-        <v>298</v>
+        <v>293</v>
       </c>
       <c r="D215" s="3" t="n">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="E215" s="3" t="inlineStr">
         <is>
@@ -7176,10 +7176,10 @@
         <v>245</v>
       </c>
       <c r="C216" s="11" t="n">
-        <v>178</v>
+        <v>163</v>
       </c>
       <c r="D216" s="3" t="n">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E216" s="3" t="inlineStr">
         <is>
@@ -7206,11 +7206,11 @@
       <c r="B217" s="3" t="n">
         <v>246</v>
       </c>
-      <c r="C217" s="5" t="n">
-        <v>281</v>
+      <c r="C217" s="4" t="n">
+        <v>288</v>
       </c>
       <c r="D217" s="3" t="n">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="E217" s="3" t="inlineStr">
         <is>
@@ -7238,10 +7238,10 @@
         <v>248</v>
       </c>
       <c r="C218" s="5" t="n">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D218" s="3" t="n">
-        <v>225</v>
+        <v>212</v>
       </c>
       <c r="E218" s="3" t="inlineStr">
         <is>
@@ -7269,10 +7269,10 @@
         <v>249</v>
       </c>
       <c r="C219" s="5" t="n">
-        <v>277</v>
+        <v>204</v>
       </c>
       <c r="D219" s="3" t="n">
-        <v>204</v>
+        <v>210</v>
       </c>
       <c r="E219" s="3" t="inlineStr">
         <is>
@@ -7300,7 +7300,7 @@
         <v>250</v>
       </c>
       <c r="C220" s="4" t="n">
-        <v>301</v>
+        <v>295</v>
       </c>
       <c r="D220" s="3" t="inlineStr"/>
       <c r="E220" s="3" t="inlineStr">
@@ -7329,10 +7329,10 @@
         <v>251</v>
       </c>
       <c r="C221" s="5" t="n">
-        <v>285</v>
+        <v>203</v>
       </c>
       <c r="D221" s="3" t="n">
-        <v>271</v>
+        <v>208</v>
       </c>
       <c r="E221" s="3" t="inlineStr">
         <is>
@@ -7360,10 +7360,10 @@
         <v>252</v>
       </c>
       <c r="C222" s="5" t="n">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="D222" s="3" t="n">
-        <v>270</v>
+        <v>276</v>
       </c>
       <c r="E222" s="3" t="inlineStr">
         <is>
@@ -7391,10 +7391,10 @@
         <v>254</v>
       </c>
       <c r="C223" s="5" t="n">
-        <v>233</v>
+        <v>258</v>
       </c>
       <c r="D223" s="3" t="n">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="E223" s="3" t="inlineStr">
         <is>
@@ -7451,10 +7451,10 @@
         <v>256</v>
       </c>
       <c r="C225" s="5" t="n">
-        <v>261</v>
+        <v>236</v>
       </c>
       <c r="D225" s="3" t="n">
-        <v>294</v>
+        <v>232</v>
       </c>
       <c r="E225" s="3" t="inlineStr">
         <is>
@@ -7482,10 +7482,10 @@
         <v>257</v>
       </c>
       <c r="C226" s="5" t="n">
-        <v>274</v>
+        <v>287</v>
       </c>
       <c r="D226" s="3" t="n">
-        <v>275</v>
+        <v>279</v>
       </c>
       <c r="E226" s="3" t="inlineStr">
         <is>
@@ -7513,7 +7513,7 @@
         <v>258</v>
       </c>
       <c r="C227" s="4" t="n">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="D227" s="3" t="inlineStr"/>
       <c r="E227" s="3" t="inlineStr">
@@ -7542,11 +7542,9 @@
         <v>259</v>
       </c>
       <c r="C228" s="5" t="n">
-        <v>281</v>
-      </c>
-      <c r="D228" s="3" t="n">
-        <v>301</v>
-      </c>
+        <v>277</v>
+      </c>
+      <c r="D228" s="3" t="inlineStr"/>
       <c r="E228" s="3" t="inlineStr">
         <is>
           <t>Eli Stowers</t>
@@ -7573,10 +7571,10 @@
         <v>260</v>
       </c>
       <c r="C229" s="5" t="n">
-        <v>272</v>
+        <v>280</v>
       </c>
       <c r="D229" s="3" t="n">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E229" s="3" t="inlineStr">
         <is>
@@ -7604,10 +7602,10 @@
         <v>261</v>
       </c>
       <c r="C230" s="4" t="n">
-        <v>306</v>
+        <v>311</v>
       </c>
       <c r="D230" s="3" t="n">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="E230" s="3" t="inlineStr">
         <is>
@@ -7634,11 +7632,11 @@
       <c r="B231" s="3" t="n">
         <v>262</v>
       </c>
-      <c r="C231" s="5" t="n">
-        <v>203</v>
+      <c r="C231" s="11" t="n">
+        <v>196</v>
       </c>
       <c r="D231" s="3" t="n">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="E231" s="3" t="inlineStr">
         <is>
@@ -7669,7 +7667,7 @@
         <v>261</v>
       </c>
       <c r="D232" s="3" t="n">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="E232" s="3" t="inlineStr">
         <is>
@@ -7697,10 +7695,10 @@
         <v>265</v>
       </c>
       <c r="C233" s="5" t="n">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="D233" s="3" t="n">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="E233" s="3" t="inlineStr">
         <is>
@@ -7728,10 +7726,10 @@
         <v>266</v>
       </c>
       <c r="C234" s="5" t="n">
-        <v>241</v>
+        <v>252</v>
       </c>
       <c r="D234" s="3" t="n">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="E234" s="3" t="inlineStr">
         <is>
@@ -7759,10 +7757,10 @@
         <v>267</v>
       </c>
       <c r="C235" s="5" t="n">
-        <v>236</v>
+        <v>256</v>
       </c>
       <c r="D235" s="3" t="n">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="E235" s="3" t="inlineStr">
         <is>
@@ -7790,7 +7788,7 @@
         <v>268</v>
       </c>
       <c r="C236" s="4" t="n">
-        <v>340</v>
+        <v>319</v>
       </c>
       <c r="D236" s="3" t="inlineStr"/>
       <c r="E236" s="3" t="inlineStr">
@@ -7819,10 +7817,10 @@
         <v>269</v>
       </c>
       <c r="C237" s="5" t="n">
-        <v>209</v>
+        <v>238</v>
       </c>
       <c r="D237" s="3" t="n">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="E237" s="3" t="inlineStr">
         <is>
@@ -7850,10 +7848,10 @@
         <v>270</v>
       </c>
       <c r="C238" s="5" t="n">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D238" s="3" t="n">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="E238" s="3" t="inlineStr">
         <is>
@@ -7881,10 +7879,10 @@
         <v>271</v>
       </c>
       <c r="C239" s="5" t="n">
-        <v>255</v>
+        <v>299</v>
       </c>
       <c r="D239" s="3" t="n">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="E239" s="3" t="inlineStr">
         <is>
@@ -7912,10 +7910,10 @@
         <v>272</v>
       </c>
       <c r="C240" s="5" t="n">
-        <v>293</v>
+        <v>288</v>
       </c>
       <c r="D240" s="3" t="n">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="E240" s="3" t="inlineStr">
         <is>
@@ -7942,8 +7940,8 @@
       <c r="B241" s="3" t="n">
         <v>273</v>
       </c>
-      <c r="C241" s="5" t="n">
-        <v>313</v>
+      <c r="C241" s="4" t="n">
+        <v>341</v>
       </c>
       <c r="D241" s="3" t="inlineStr"/>
       <c r="E241" s="3" t="inlineStr">
@@ -7972,7 +7970,7 @@
         <v>274</v>
       </c>
       <c r="C242" s="5" t="n">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="D242" s="3" t="inlineStr"/>
       <c r="E242" s="3" t="inlineStr">
@@ -8001,7 +7999,7 @@
         <v>275</v>
       </c>
       <c r="C243" s="5" t="n">
-        <v>283</v>
+        <v>279</v>
       </c>
       <c r="D243" s="3" t="inlineStr"/>
       <c r="E243" s="3" t="inlineStr">
@@ -8033,7 +8031,7 @@
         <v>275</v>
       </c>
       <c r="D244" s="3" t="n">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="E244" s="3" t="inlineStr">
         <is>
@@ -8061,10 +8059,10 @@
         <v>277</v>
       </c>
       <c r="C245" s="5" t="n">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D245" s="3" t="n">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="E245" s="3" t="inlineStr">
         <is>
@@ -8091,11 +8089,11 @@
       <c r="B246" s="3" t="n">
         <v>278</v>
       </c>
-      <c r="C246" s="11" t="n">
-        <v>193</v>
+      <c r="C246" s="5" t="n">
+        <v>219</v>
       </c>
       <c r="D246" s="3" t="n">
-        <v>223</v>
+        <v>206</v>
       </c>
       <c r="E246" s="3" t="inlineStr">
         <is>
@@ -8123,7 +8121,7 @@
         <v>280</v>
       </c>
       <c r="C247" s="4" t="n">
-        <v>348</v>
+        <v>354</v>
       </c>
       <c r="D247" s="3" t="inlineStr"/>
       <c r="E247" s="3" t="inlineStr">
@@ -8152,7 +8150,7 @@
         <v>281</v>
       </c>
       <c r="C248" s="5" t="n">
-        <v>292</v>
+        <v>285</v>
       </c>
       <c r="D248" s="3" t="inlineStr"/>
       <c r="E248" s="3" t="inlineStr">
@@ -8181,10 +8179,10 @@
         <v>282</v>
       </c>
       <c r="C249" s="5" t="n">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="D249" s="3" t="n">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="E249" s="3" t="inlineStr">
         <is>
@@ -8212,10 +8210,10 @@
         <v>283</v>
       </c>
       <c r="C250" s="5" t="n">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D250" s="3" t="n">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="E250" s="3" t="inlineStr">
         <is>
@@ -8243,7 +8241,7 @@
         <v>284</v>
       </c>
       <c r="C251" s="5" t="n">
-        <v>312</v>
+        <v>287</v>
       </c>
       <c r="D251" s="3" t="inlineStr"/>
       <c r="E251" s="3" t="inlineStr">
@@ -8272,10 +8270,10 @@
         <v>285</v>
       </c>
       <c r="C252" s="5" t="n">
-        <v>290</v>
+        <v>264</v>
       </c>
       <c r="D252" s="3" t="n">
-        <v>300</v>
+        <v>218</v>
       </c>
       <c r="E252" s="3" t="inlineStr">
         <is>
@@ -8303,7 +8301,7 @@
         <v>288</v>
       </c>
       <c r="C253" s="4" t="n">
-        <v>345</v>
+        <v>340</v>
       </c>
       <c r="D253" s="3" t="inlineStr"/>
       <c r="E253" s="3" t="inlineStr">
@@ -8332,7 +8330,7 @@
         <v>289</v>
       </c>
       <c r="C254" s="5" t="n">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="D254" s="3" t="inlineStr"/>
       <c r="E254" s="3" t="inlineStr">
@@ -8361,10 +8359,10 @@
         <v>290</v>
       </c>
       <c r="C255" s="5" t="n">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="D255" s="3" t="n">
-        <v>251</v>
+        <v>147</v>
       </c>
       <c r="E255" s="3" t="inlineStr">
         <is>
@@ -8391,8 +8389,8 @@
       <c r="B256" s="3" t="n">
         <v>292</v>
       </c>
-      <c r="C256" s="5" t="n">
-        <v>335</v>
+      <c r="C256" s="4" t="n">
+        <v>337</v>
       </c>
       <c r="D256" s="3" t="inlineStr"/>
       <c r="E256" s="3" t="inlineStr">
@@ -8424,7 +8422,7 @@
         <v>239</v>
       </c>
       <c r="D257" s="3" t="n">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="E257" s="3" t="inlineStr">
         <is>
@@ -8452,7 +8450,7 @@
         <v>294</v>
       </c>
       <c r="C258" s="4" t="n">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="D258" s="3" t="inlineStr"/>
       <c r="E258" s="3" t="inlineStr">
@@ -8481,7 +8479,7 @@
         <v>296</v>
       </c>
       <c r="C259" s="5" t="n">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="D259" s="3" t="inlineStr"/>
       <c r="E259" s="3" t="inlineStr">
@@ -8510,7 +8508,7 @@
         <v>297</v>
       </c>
       <c r="C260" s="5" t="n">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="D260" s="3" t="inlineStr"/>
       <c r="E260" s="3" t="inlineStr">
@@ -8539,10 +8537,10 @@
         <v>298</v>
       </c>
       <c r="C261" s="5" t="n">
-        <v>287</v>
+        <v>274</v>
       </c>
       <c r="D261" s="3" t="n">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="E261" s="3" t="inlineStr">
         <is>
@@ -8570,10 +8568,10 @@
         <v>299</v>
       </c>
       <c r="C262" s="5" t="n">
-        <v>252</v>
+        <v>241</v>
       </c>
       <c r="D262" s="3" t="n">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="E262" s="3" t="inlineStr">
         <is>
@@ -8604,7 +8602,7 @@
         <v>280</v>
       </c>
       <c r="D263" s="3" t="n">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="E263" s="3" t="inlineStr">
         <is>
@@ -8631,8 +8629,8 @@
       <c r="B264" s="3" t="n">
         <v>301</v>
       </c>
-      <c r="C264" s="5" t="n">
-        <v>323</v>
+      <c r="C264" s="4" t="n">
+        <v>367</v>
       </c>
       <c r="D264" s="3" t="inlineStr"/>
       <c r="E264" s="3" t="inlineStr">
@@ -8664,7 +8662,7 @@
         <v>253</v>
       </c>
       <c r="D265" s="3" t="n">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="E265" s="3" t="inlineStr">
         <is>
@@ -8692,7 +8690,7 @@
         <v>304</v>
       </c>
       <c r="C266" s="5" t="n">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="D266" s="3" t="inlineStr"/>
       <c r="E266" s="3" t="inlineStr">
@@ -8721,7 +8719,7 @@
         <v>305</v>
       </c>
       <c r="C267" s="5" t="n">
-        <v>287</v>
+        <v>281</v>
       </c>
       <c r="D267" s="3" t="inlineStr"/>
       <c r="E267" s="3" t="inlineStr">
@@ -8750,10 +8748,10 @@
         <v>306</v>
       </c>
       <c r="C268" s="11" t="n">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="D268" s="3" t="n">
-        <v>202</v>
+        <v>181</v>
       </c>
       <c r="E268" s="3" t="inlineStr">
         <is>
@@ -8781,7 +8779,7 @@
         <v>309</v>
       </c>
       <c r="C269" s="5" t="n">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="D269" s="3" t="inlineStr"/>
       <c r="E269" s="3" t="inlineStr">
@@ -8810,7 +8808,7 @@
         <v>310</v>
       </c>
       <c r="C270" s="5" t="n">
-        <v>305</v>
+        <v>316</v>
       </c>
       <c r="D270" s="3" t="inlineStr"/>
       <c r="E270" s="3" t="inlineStr">
@@ -8839,7 +8837,7 @@
         <v>311</v>
       </c>
       <c r="C271" s="5" t="n">
-        <v>294</v>
+        <v>320</v>
       </c>
       <c r="D271" s="3" t="inlineStr"/>
       <c r="E271" s="3" t="inlineStr">
@@ -8868,7 +8866,7 @@
         <v>312</v>
       </c>
       <c r="C272" s="5" t="n">
-        <v>333</v>
+        <v>312</v>
       </c>
       <c r="D272" s="3" t="inlineStr"/>
       <c r="E272" s="3" t="inlineStr">
@@ -8897,7 +8895,7 @@
         <v>314</v>
       </c>
       <c r="C273" s="5" t="n">
-        <v>297</v>
+        <v>306</v>
       </c>
       <c r="D273" s="3" t="inlineStr"/>
       <c r="E273" s="3" t="inlineStr">
@@ -8926,10 +8924,10 @@
         <v>316</v>
       </c>
       <c r="C274" s="5" t="n">
-        <v>255</v>
+        <v>262</v>
       </c>
       <c r="D274" s="3" t="n">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="E274" s="3" t="inlineStr">
         <is>
@@ -8957,7 +8955,7 @@
         <v>317</v>
       </c>
       <c r="C275" s="5" t="n">
-        <v>296</v>
+        <v>352</v>
       </c>
       <c r="D275" s="3" t="inlineStr"/>
       <c r="E275" s="3" t="inlineStr">
@@ -8977,88 +8975,86 @@
       </c>
     </row>
     <row r="276">
-      <c r="A276" s="8" t="inlineStr">
+      <c r="A276" s="6" t="inlineStr">
+        <is>
+          <t>RB98</t>
+        </is>
+      </c>
+      <c r="B276" s="3" t="n">
+        <v>321</v>
+      </c>
+      <c r="C276" s="5" t="n">
+        <v>348</v>
+      </c>
+      <c r="D276" s="3" t="inlineStr"/>
+      <c r="E276" s="3" t="inlineStr">
+        <is>
+          <t>Audric Estime</t>
+        </is>
+      </c>
+      <c r="F276" s="3" t="inlineStr">
+        <is>
+          <t>NO (8)</t>
+        </is>
+      </c>
+      <c r="G276" s="3" t="inlineStr">
+        <is>
+          <t>RB</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="8" t="inlineStr">
         <is>
           <t>TE39</t>
         </is>
       </c>
-      <c r="B276" s="3" t="n">
+      <c r="B277" s="3" t="n">
         <v>322</v>
       </c>
-      <c r="C276" s="5" t="n">
+      <c r="C277" s="5" t="n">
         <v>282</v>
       </c>
-      <c r="D276" s="3" t="n">
-        <v>272</v>
-      </c>
-      <c r="E276" s="3" t="inlineStr">
+      <c r="D277" s="3" t="n">
+        <v>277</v>
+      </c>
+      <c r="E277" s="3" t="inlineStr">
         <is>
           <t>Darnell Washington</t>
         </is>
       </c>
-      <c r="F276" s="3" t="inlineStr">
+      <c r="F277" s="3" t="inlineStr">
         <is>
           <t>PIT (9)</t>
         </is>
       </c>
-      <c r="G276" s="3" t="inlineStr">
+      <c r="G277" s="3" t="inlineStr">
         <is>
           <t>TE</t>
-        </is>
-      </c>
-    </row>
-    <row r="277">
-      <c r="A277" s="10" t="inlineStr">
-        <is>
-          <t>QB36</t>
-        </is>
-      </c>
-      <c r="B277" s="3" t="n">
-        <v>327</v>
-      </c>
-      <c r="C277" s="5" t="n">
-        <v>368</v>
-      </c>
-      <c r="D277" s="3" t="inlineStr"/>
-      <c r="E277" s="3" t="inlineStr">
-        <is>
-          <t>J.J. McCarthy</t>
-        </is>
-      </c>
-      <c r="F277" s="3" t="inlineStr">
-        <is>
-          <t>MIN (6)</t>
-        </is>
-      </c>
-      <c r="G277" s="3" t="inlineStr">
-        <is>
-          <t>QB</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" s="2" t="inlineStr">
         <is>
-          <t>WR114</t>
+          <t>WR112</t>
         </is>
       </c>
       <c r="B278" s="3" t="n">
-        <v>328</v>
-      </c>
-      <c r="C278" s="5" t="n">
-        <v>284</v>
-      </c>
-      <c r="D278" s="3" t="n">
-        <v>266</v>
-      </c>
+        <v>324</v>
+      </c>
+      <c r="C278" s="4" t="n">
+        <v>375</v>
+      </c>
+      <c r="D278" s="3" t="inlineStr"/>
       <c r="E278" s="3" t="inlineStr">
         <is>
-          <t>Luke McCaffrey</t>
+          <t>Cedric Tillman</t>
         </is>
       </c>
       <c r="F278" s="3" t="inlineStr">
         <is>
-          <t>WAS (7)</t>
+          <t>CLE (11)</t>
         </is>
       </c>
       <c r="G278" s="3" t="inlineStr">
@@ -9068,55 +9064,57 @@
       </c>
     </row>
     <row r="279">
-      <c r="A279" s="2" t="inlineStr">
-        <is>
-          <t>WR116</t>
+      <c r="A279" s="10" t="inlineStr">
+        <is>
+          <t>QB36</t>
         </is>
       </c>
       <c r="B279" s="3" t="n">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="C279" s="5" t="n">
-        <v>266</v>
+        <v>369</v>
       </c>
       <c r="D279" s="3" t="inlineStr"/>
       <c r="E279" s="3" t="inlineStr">
         <is>
-          <t>Jahan Dotson</t>
+          <t>J.J. McCarthy</t>
         </is>
       </c>
       <c r="F279" s="3" t="inlineStr">
         <is>
-          <t>ATL (11)</t>
+          <t>MIN (6)</t>
         </is>
       </c>
       <c r="G279" s="3" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>QB</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" s="2" t="inlineStr">
         <is>
-          <t>WR117</t>
+          <t>WR114</t>
         </is>
       </c>
       <c r="B280" s="3" t="n">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="C280" s="5" t="n">
-        <v>352</v>
-      </c>
-      <c r="D280" s="3" t="inlineStr"/>
+        <v>294</v>
+      </c>
+      <c r="D280" s="3" t="n">
+        <v>270</v>
+      </c>
       <c r="E280" s="3" t="inlineStr">
         <is>
-          <t>Jalen Royals</t>
+          <t>Luke McCaffrey</t>
         </is>
       </c>
       <c r="F280" s="3" t="inlineStr">
         <is>
-          <t>KC (5)</t>
+          <t>WAS (7)</t>
         </is>
       </c>
       <c r="G280" s="3" t="inlineStr">
@@ -9126,13 +9124,13 @@
       </c>
     </row>
     <row r="281">
-      <c r="A281" s="8" t="inlineStr">
-        <is>
-          <t>TE40</t>
+      <c r="A281" s="2" t="inlineStr">
+        <is>
+          <t>WR115</t>
         </is>
       </c>
       <c r="B281" s="3" t="n">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="C281" s="5" t="n">
         <v>370</v>
@@ -9140,43 +9138,41 @@
       <c r="D281" s="3" t="inlineStr"/>
       <c r="E281" s="3" t="inlineStr">
         <is>
-          <t>Max Klare</t>
+          <t>Tez Johnson</t>
         </is>
       </c>
       <c r="F281" s="3" t="inlineStr">
         <is>
-          <t>LAR (11)</t>
+          <t>TB (10)</t>
         </is>
       </c>
       <c r="G281" s="3" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>WR</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" s="2" t="inlineStr">
         <is>
-          <t>WR118</t>
+          <t>WR116</t>
         </is>
       </c>
       <c r="B282" s="3" t="n">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="C282" s="5" t="n">
-        <v>201</v>
-      </c>
-      <c r="D282" s="3" t="n">
-        <v>207</v>
-      </c>
+        <v>269</v>
+      </c>
+      <c r="D282" s="3" t="inlineStr"/>
       <c r="E282" s="3" t="inlineStr">
         <is>
-          <t>Caleb Douglas</t>
+          <t>Jahan Dotson</t>
         </is>
       </c>
       <c r="F282" s="3" t="inlineStr">
         <is>
-          <t>MIA (6)</t>
+          <t>ATL (11)</t>
         </is>
       </c>
       <c r="G282" s="3" t="inlineStr">
@@ -9188,26 +9184,24 @@
     <row r="283">
       <c r="A283" s="2" t="inlineStr">
         <is>
-          <t>WR120</t>
+          <t>WR117</t>
         </is>
       </c>
       <c r="B283" s="3" t="n">
-        <v>335</v>
+        <v>331</v>
       </c>
       <c r="C283" s="5" t="n">
-        <v>297</v>
-      </c>
-      <c r="D283" s="3" t="n">
-        <v>280</v>
-      </c>
+        <v>347</v>
+      </c>
+      <c r="D283" s="3" t="inlineStr"/>
       <c r="E283" s="3" t="inlineStr">
         <is>
-          <t>Jalen Tolbert</t>
+          <t>Jalen Royals</t>
         </is>
       </c>
       <c r="F283" s="3" t="inlineStr">
         <is>
-          <t>MIA (6)</t>
+          <t>KC (5)</t>
         </is>
       </c>
       <c r="G283" s="3" t="inlineStr">
@@ -9217,171 +9211,177 @@
       </c>
     </row>
     <row r="284">
-      <c r="A284" s="2" t="inlineStr">
-        <is>
-          <t>WR122</t>
+      <c r="A284" s="8" t="inlineStr">
+        <is>
+          <t>TE40</t>
         </is>
       </c>
       <c r="B284" s="3" t="n">
-        <v>337</v>
+        <v>332</v>
       </c>
       <c r="C284" s="5" t="n">
-        <v>353</v>
+        <v>374</v>
       </c>
       <c r="D284" s="3" t="inlineStr"/>
       <c r="E284" s="3" t="inlineStr">
         <is>
-          <t>Joshua Palmer</t>
+          <t>Max Klare</t>
         </is>
       </c>
       <c r="F284" s="3" t="inlineStr">
         <is>
-          <t>BUF (7)</t>
+          <t>LAR (11)</t>
         </is>
       </c>
       <c r="G284" s="3" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>TE</t>
         </is>
       </c>
     </row>
     <row r="285">
-      <c r="A285" s="8" t="inlineStr">
-        <is>
-          <t>TE41</t>
+      <c r="A285" s="2" t="inlineStr">
+        <is>
+          <t>WR118</t>
         </is>
       </c>
       <c r="B285" s="3" t="n">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="C285" s="5" t="n">
-        <v>362</v>
-      </c>
-      <c r="D285" s="3" t="inlineStr"/>
+        <v>224</v>
+      </c>
+      <c r="D285" s="3" t="n">
+        <v>209</v>
+      </c>
       <c r="E285" s="3" t="inlineStr">
         <is>
-          <t>Michael Mayer</t>
+          <t>Caleb Douglas</t>
         </is>
       </c>
       <c r="F285" s="3" t="inlineStr">
         <is>
-          <t>LV (13)</t>
+          <t>MIA (6)</t>
         </is>
       </c>
       <c r="G285" s="3" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>WR</t>
         </is>
       </c>
     </row>
     <row r="286">
-      <c r="A286" s="8" t="inlineStr">
-        <is>
-          <t>TE42</t>
+      <c r="A286" s="2" t="inlineStr">
+        <is>
+          <t>WR119</t>
         </is>
       </c>
       <c r="B286" s="3" t="n">
-        <v>340</v>
+        <v>334</v>
       </c>
       <c r="C286" s="5" t="n">
-        <v>330</v>
-      </c>
-      <c r="D286" s="3" t="inlineStr"/>
+        <v>286</v>
+      </c>
+      <c r="D286" s="3" t="n">
+        <v>269</v>
+      </c>
       <c r="E286" s="3" t="inlineStr">
         <is>
-          <t>Elijah Arroyo</t>
+          <t>Calvin Austin</t>
         </is>
       </c>
       <c r="F286" s="3" t="inlineStr">
         <is>
-          <t>SEA (11)</t>
+          <t>NYG (8)</t>
         </is>
       </c>
       <c r="G286" s="3" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>WR</t>
         </is>
       </c>
     </row>
     <row r="287">
-      <c r="A287" s="8" t="inlineStr">
-        <is>
-          <t>TE43</t>
+      <c r="A287" s="2" t="inlineStr">
+        <is>
+          <t>WR120</t>
         </is>
       </c>
       <c r="B287" s="3" t="n">
-        <v>341</v>
+        <v>335</v>
       </c>
       <c r="C287" s="5" t="n">
-        <v>307</v>
-      </c>
-      <c r="D287" s="3" t="inlineStr"/>
+        <v>359</v>
+      </c>
+      <c r="D287" s="3" t="n">
+        <v>299</v>
+      </c>
       <c r="E287" s="3" t="inlineStr">
         <is>
-          <t>Tyler Higbee</t>
+          <t>Jalen Tolbert</t>
         </is>
       </c>
       <c r="F287" s="3" t="inlineStr">
         <is>
-          <t>LAR (11)</t>
+          <t>MIA (6)</t>
         </is>
       </c>
       <c r="G287" s="3" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>WR</t>
         </is>
       </c>
     </row>
     <row r="288">
-      <c r="A288" s="10" t="inlineStr">
-        <is>
-          <t>QB37</t>
+      <c r="A288" s="2" t="inlineStr">
+        <is>
+          <t>WR122</t>
         </is>
       </c>
       <c r="B288" s="3" t="n">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="C288" s="5" t="n">
-        <v>372</v>
+        <v>331</v>
       </c>
       <c r="D288" s="3" t="inlineStr"/>
       <c r="E288" s="3" t="inlineStr">
         <is>
-          <t>Mac Jones</t>
+          <t>Joshua Palmer</t>
         </is>
       </c>
       <c r="F288" s="3" t="inlineStr">
         <is>
-          <t>SF (8)</t>
+          <t>BUF (7)</t>
         </is>
       </c>
       <c r="G288" s="3" t="inlineStr">
         <is>
-          <t>QB</t>
+          <t>WR</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" s="8" t="inlineStr">
         <is>
-          <t>TE45</t>
+          <t>TE41</t>
         </is>
       </c>
       <c r="B289" s="3" t="n">
-        <v>344</v>
+        <v>338</v>
       </c>
       <c r="C289" s="5" t="n">
-        <v>367</v>
+        <v>328</v>
       </c>
       <c r="D289" s="3" t="inlineStr"/>
       <c r="E289" s="3" t="inlineStr">
         <is>
-          <t>Dawson Knox</t>
+          <t>Michael Mayer</t>
         </is>
       </c>
       <c r="F289" s="3" t="inlineStr">
         <is>
-          <t>BUF (7)</t>
+          <t>LV (13)</t>
         </is>
       </c>
       <c r="G289" s="3" t="inlineStr">
@@ -9391,55 +9391,55 @@
       </c>
     </row>
     <row r="290">
-      <c r="A290" s="10" t="inlineStr">
-        <is>
-          <t>QB38</t>
+      <c r="A290" s="8" t="inlineStr">
+        <is>
+          <t>TE42</t>
         </is>
       </c>
       <c r="B290" s="3" t="n">
-        <v>348</v>
+        <v>340</v>
       </c>
       <c r="C290" s="5" t="n">
-        <v>342</v>
+        <v>335</v>
       </c>
       <c r="D290" s="3" t="inlineStr"/>
       <c r="E290" s="3" t="inlineStr">
         <is>
-          <t>Carson Beck</t>
+          <t>Elijah Arroyo</t>
         </is>
       </c>
       <c r="F290" s="3" t="inlineStr">
         <is>
-          <t>ARI (14)</t>
+          <t>SEA (11)</t>
         </is>
       </c>
       <c r="G290" s="3" t="inlineStr">
         <is>
-          <t>QB</t>
+          <t>TE</t>
         </is>
       </c>
     </row>
     <row r="291">
       <c r="A291" s="8" t="inlineStr">
         <is>
-          <t>TE47</t>
+          <t>TE43</t>
         </is>
       </c>
       <c r="B291" s="3" t="n">
-        <v>349</v>
+        <v>341</v>
       </c>
       <c r="C291" s="5" t="n">
-        <v>366</v>
+        <v>310</v>
       </c>
       <c r="D291" s="3" t="inlineStr"/>
       <c r="E291" s="3" t="inlineStr">
         <is>
-          <t>Cole Kmet</t>
+          <t>Tyler Higbee</t>
         </is>
       </c>
       <c r="F291" s="3" t="inlineStr">
         <is>
-          <t>CHI (10)</t>
+          <t>LAR (11)</t>
         </is>
       </c>
       <c r="G291" s="3" t="inlineStr">
@@ -9449,144 +9449,142 @@
       </c>
     </row>
     <row r="292">
-      <c r="A292" s="2" t="inlineStr">
-        <is>
-          <t>WR124</t>
+      <c r="A292" s="10" t="inlineStr">
+        <is>
+          <t>QB37</t>
         </is>
       </c>
       <c r="B292" s="3" t="n">
-        <v>350</v>
+        <v>342</v>
       </c>
       <c r="C292" s="5" t="n">
-        <v>331</v>
+        <v>378</v>
       </c>
       <c r="D292" s="3" t="inlineStr"/>
       <c r="E292" s="3" t="inlineStr">
         <is>
-          <t>Brenen Thompson</t>
+          <t>Mac Jones</t>
         </is>
       </c>
       <c r="F292" s="3" t="inlineStr">
         <is>
-          <t>LAC (7)</t>
+          <t>SF (8)</t>
         </is>
       </c>
       <c r="G292" s="3" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>QB</t>
         </is>
       </c>
     </row>
     <row r="293">
-      <c r="A293" s="2" t="inlineStr">
-        <is>
-          <t>WR125</t>
+      <c r="A293" s="8" t="inlineStr">
+        <is>
+          <t>TE45</t>
         </is>
       </c>
       <c r="B293" s="3" t="n">
-        <v>351</v>
+        <v>344</v>
       </c>
       <c r="C293" s="5" t="n">
-        <v>339</v>
+        <v>376</v>
       </c>
       <c r="D293" s="3" t="inlineStr"/>
       <c r="E293" s="3" t="inlineStr">
         <is>
-          <t>DeMario Douglas</t>
+          <t>Dawson Knox</t>
         </is>
       </c>
       <c r="F293" s="3" t="inlineStr">
         <is>
-          <t>NE (11)</t>
+          <t>BUF (7)</t>
         </is>
       </c>
       <c r="G293" s="3" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>TE</t>
         </is>
       </c>
     </row>
     <row r="294">
-      <c r="A294" s="6" t="inlineStr">
-        <is>
-          <t>RB104</t>
+      <c r="A294" s="10" t="inlineStr">
+        <is>
+          <t>QB38</t>
         </is>
       </c>
       <c r="B294" s="3" t="n">
-        <v>360</v>
+        <v>348</v>
       </c>
       <c r="C294" s="5" t="n">
-        <v>351</v>
+        <v>342</v>
       </c>
       <c r="D294" s="3" t="inlineStr"/>
       <c r="E294" s="3" t="inlineStr">
         <is>
-          <t>Jawhar Jordan</t>
+          <t>Carson Beck</t>
         </is>
       </c>
       <c r="F294" s="3" t="inlineStr">
         <is>
-          <t>HOU (8)</t>
+          <t>ARI (14)</t>
         </is>
       </c>
       <c r="G294" s="3" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>QB</t>
         </is>
       </c>
     </row>
     <row r="295">
-      <c r="A295" s="2" t="inlineStr">
-        <is>
-          <t>WR130</t>
+      <c r="A295" s="8" t="inlineStr">
+        <is>
+          <t>TE47</t>
         </is>
       </c>
       <c r="B295" s="3" t="n">
-        <v>363</v>
+        <v>349</v>
       </c>
       <c r="C295" s="5" t="n">
-        <v>338</v>
-      </c>
-      <c r="D295" s="3" t="n">
-        <v>293</v>
-      </c>
+        <v>371</v>
+      </c>
+      <c r="D295" s="3" t="inlineStr"/>
       <c r="E295" s="3" t="inlineStr">
         <is>
-          <t>Treylon Burks</t>
+          <t>Cole Kmet</t>
         </is>
       </c>
       <c r="F295" s="3" t="inlineStr">
         <is>
-          <t>WAS (7)</t>
+          <t>CHI (10)</t>
         </is>
       </c>
       <c r="G295" s="3" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>TE</t>
         </is>
       </c>
     </row>
     <row r="296">
       <c r="A296" s="2" t="inlineStr">
         <is>
-          <t>WR133</t>
+          <t>WR124</t>
         </is>
       </c>
       <c r="B296" s="3" t="n">
-        <v>367</v>
+        <v>350</v>
       </c>
       <c r="C296" s="5" t="n">
-        <v>358</v>
+        <v>339</v>
       </c>
       <c r="D296" s="3" t="inlineStr"/>
       <c r="E296" s="3" t="inlineStr">
         <is>
-          <t>Savion Williams</t>
+          <t>Brenen Thompson</t>
         </is>
       </c>
       <c r="F296" s="3" t="inlineStr">
         <is>
-          <t>GB (11)</t>
+          <t>LAC (7)</t>
         </is>
       </c>
       <c r="G296" s="3" t="inlineStr">
@@ -9596,55 +9594,55 @@
       </c>
     </row>
     <row r="297">
-      <c r="A297" s="8" t="inlineStr">
-        <is>
-          <t>TE49</t>
+      <c r="A297" s="2" t="inlineStr">
+        <is>
+          <t>WR125</t>
         </is>
       </c>
       <c r="B297" s="3" t="n">
-        <v>373</v>
+        <v>351</v>
       </c>
       <c r="C297" s="5" t="n">
-        <v>371</v>
+        <v>326</v>
       </c>
       <c r="D297" s="3" t="inlineStr"/>
       <c r="E297" s="3" t="inlineStr">
         <is>
-          <t>Noah Fant</t>
+          <t>DeMario Douglas</t>
         </is>
       </c>
       <c r="F297" s="3" t="inlineStr">
         <is>
-          <t>NO (8)</t>
+          <t>NE (11)</t>
         </is>
       </c>
       <c r="G297" s="3" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>WR</t>
         </is>
       </c>
     </row>
     <row r="298">
       <c r="A298" s="6" t="inlineStr">
         <is>
-          <t>RB107</t>
+          <t>RB104</t>
         </is>
       </c>
       <c r="B298" s="3" t="n">
-        <v>374</v>
+        <v>360</v>
       </c>
       <c r="C298" s="5" t="n">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="D298" s="3" t="inlineStr"/>
       <c r="E298" s="3" t="inlineStr">
         <is>
-          <t>Raheim Sanders</t>
+          <t>Jawhar Jordan</t>
         </is>
       </c>
       <c r="F298" s="3" t="inlineStr">
         <is>
-          <t>CLE (11)</t>
+          <t>HOU (8)</t>
         </is>
       </c>
       <c r="G298" s="3" t="inlineStr">
@@ -9654,55 +9652,57 @@
       </c>
     </row>
     <row r="299">
-      <c r="A299" s="8" t="inlineStr">
-        <is>
-          <t>TE50</t>
+      <c r="A299" s="2" t="inlineStr">
+        <is>
+          <t>WR130</t>
         </is>
       </c>
       <c r="B299" s="3" t="n">
-        <v>377</v>
+        <v>363</v>
       </c>
       <c r="C299" s="5" t="n">
-        <v>337</v>
-      </c>
-      <c r="D299" s="3" t="inlineStr"/>
+        <v>338</v>
+      </c>
+      <c r="D299" s="3" t="n">
+        <v>294</v>
+      </c>
       <c r="E299" s="3" t="inlineStr">
         <is>
-          <t>Eli Raridon</t>
+          <t>Treylon Burks</t>
         </is>
       </c>
       <c r="F299" s="3" t="inlineStr">
         <is>
-          <t>NE (11)</t>
+          <t>WAS (7)</t>
         </is>
       </c>
       <c r="G299" s="3" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>WR</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" s="2" t="inlineStr">
         <is>
-          <t>WR138</t>
+          <t>WR132</t>
         </is>
       </c>
       <c r="B300" s="3" t="n">
-        <v>383</v>
+        <v>365</v>
       </c>
       <c r="C300" s="5" t="n">
-        <v>359</v>
+        <v>373</v>
       </c>
       <c r="D300" s="3" t="inlineStr"/>
       <c r="E300" s="3" t="inlineStr">
         <is>
-          <t>Zavion Thomas</t>
+          <t>Nick Westbrook-Ikhine</t>
         </is>
       </c>
       <c r="F300" s="3" t="inlineStr">
         <is>
-          <t>CHI (10)</t>
+          <t>IND (13)</t>
         </is>
       </c>
       <c r="G300" s="3" t="inlineStr">
@@ -9712,89 +9712,205 @@
       </c>
     </row>
     <row r="301">
-      <c r="A301" s="6" t="inlineStr">
-        <is>
-          <t>RB109</t>
+      <c r="A301" s="2" t="inlineStr">
+        <is>
+          <t>WR133</t>
         </is>
       </c>
       <c r="B301" s="3" t="n">
-        <v>386</v>
+        <v>367</v>
       </c>
       <c r="C301" s="5" t="n">
-        <v>317</v>
+        <v>358</v>
       </c>
       <c r="D301" s="3" t="inlineStr"/>
       <c r="E301" s="3" t="inlineStr">
         <is>
-          <t>Phil Mafah</t>
+          <t>Savion Williams</t>
         </is>
       </c>
       <c r="F301" s="3" t="inlineStr">
         <is>
-          <t>DAL (14)</t>
+          <t>GB (11)</t>
         </is>
       </c>
       <c r="G301" s="3" t="inlineStr">
         <is>
+          <t>WR</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" s="6" t="inlineStr">
+        <is>
+          <t>RB107</t>
+        </is>
+      </c>
+      <c r="B302" s="3" t="n">
+        <v>374</v>
+      </c>
+      <c r="C302" s="5" t="n">
+        <v>350</v>
+      </c>
+      <c r="D302" s="3" t="inlineStr"/>
+      <c r="E302" s="3" t="inlineStr">
+        <is>
+          <t>Raheim Sanders</t>
+        </is>
+      </c>
+      <c r="F302" s="3" t="inlineStr">
+        <is>
+          <t>CLE (11)</t>
+        </is>
+      </c>
+      <c r="G302" s="3" t="inlineStr">
+        <is>
           <t>RB</t>
         </is>
       </c>
     </row>
-    <row r="302">
-      <c r="A302" s="8" t="inlineStr">
-        <is>
-          <t>TE52</t>
-        </is>
-      </c>
-      <c r="B302" s="3" t="n">
-        <v>387</v>
-      </c>
-      <c r="C302" s="5" t="n">
-        <v>319</v>
-      </c>
-      <c r="D302" s="3" t="n">
-        <v>274</v>
-      </c>
-      <c r="E302" s="3" t="inlineStr">
-        <is>
-          <t>Erick All</t>
-        </is>
-      </c>
-      <c r="F302" s="3" t="inlineStr">
-        <is>
-          <t>CIN (6)</t>
-        </is>
-      </c>
-      <c r="G302" s="3" t="inlineStr">
-        <is>
-          <t>TE</t>
-        </is>
-      </c>
-    </row>
     <row r="303">
-      <c r="A303" s="2" t="inlineStr">
-        <is>
-          <t>WR142</t>
+      <c r="A303" s="8" t="inlineStr">
+        <is>
+          <t>TE50</t>
         </is>
       </c>
       <c r="B303" s="3" t="n">
-        <v>395</v>
+        <v>377</v>
       </c>
       <c r="C303" s="5" t="n">
-        <v>364</v>
+        <v>313</v>
       </c>
       <c r="D303" s="3" t="inlineStr"/>
       <c r="E303" s="3" t="inlineStr">
         <is>
+          <t>Eli Raridon</t>
+        </is>
+      </c>
+      <c r="F303" s="3" t="inlineStr">
+        <is>
+          <t>NE (11)</t>
+        </is>
+      </c>
+      <c r="G303" s="3" t="inlineStr">
+        <is>
+          <t>TE</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" s="2" t="inlineStr">
+        <is>
+          <t>WR138</t>
+        </is>
+      </c>
+      <c r="B304" s="3" t="n">
+        <v>383</v>
+      </c>
+      <c r="C304" s="5" t="n">
+        <v>360</v>
+      </c>
+      <c r="D304" s="3" t="inlineStr"/>
+      <c r="E304" s="3" t="inlineStr">
+        <is>
+          <t>Zavion Thomas</t>
+        </is>
+      </c>
+      <c r="F304" s="3" t="inlineStr">
+        <is>
+          <t>CHI (10)</t>
+        </is>
+      </c>
+      <c r="G304" s="3" t="inlineStr">
+        <is>
+          <t>WR</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" s="6" t="inlineStr">
+        <is>
+          <t>RB109</t>
+        </is>
+      </c>
+      <c r="B305" s="3" t="n">
+        <v>386</v>
+      </c>
+      <c r="C305" s="5" t="n">
+        <v>318</v>
+      </c>
+      <c r="D305" s="3" t="inlineStr"/>
+      <c r="E305" s="3" t="inlineStr">
+        <is>
+          <t>Phil Mafah</t>
+        </is>
+      </c>
+      <c r="F305" s="3" t="inlineStr">
+        <is>
+          <t>DAL (14)</t>
+        </is>
+      </c>
+      <c r="G305" s="3" t="inlineStr">
+        <is>
+          <t>RB</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" s="8" t="inlineStr">
+        <is>
+          <t>TE52</t>
+        </is>
+      </c>
+      <c r="B306" s="3" t="n">
+        <v>387</v>
+      </c>
+      <c r="C306" s="5" t="n">
+        <v>322</v>
+      </c>
+      <c r="D306" s="3" t="n">
+        <v>278</v>
+      </c>
+      <c r="E306" s="3" t="inlineStr">
+        <is>
+          <t>Erick All</t>
+        </is>
+      </c>
+      <c r="F306" s="3" t="inlineStr">
+        <is>
+          <t>CIN (6)</t>
+        </is>
+      </c>
+      <c r="G306" s="3" t="inlineStr">
+        <is>
+          <t>TE</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" s="2" t="inlineStr">
+        <is>
+          <t>WR142</t>
+        </is>
+      </c>
+      <c r="B307" s="3" t="n">
+        <v>395</v>
+      </c>
+      <c r="C307" s="5" t="n">
+        <v>363</v>
+      </c>
+      <c r="D307" s="3" t="inlineStr"/>
+      <c r="E307" s="3" t="inlineStr">
+        <is>
           <t>Jordan Whittington</t>
         </is>
       </c>
-      <c r="F303" s="3" t="inlineStr">
+      <c r="F307" s="3" t="inlineStr">
         <is>
           <t>LAR (11)</t>
         </is>
       </c>
-      <c r="G303" s="3" t="inlineStr">
+      <c r="G307" s="3" t="inlineStr">
         <is>
           <t>WR</t>
         </is>

</xml_diff>

<commit_message>
Refresh 2026 rankings data
</commit_message>
<xml_diff>
--- a/frontend/public/data/2026/fpros/fpros_merged_formatted.xlsx
+++ b/frontend/public/data/2026/fpros/fpros_merged_formatted.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G305"/>
+  <dimension ref="A1:G306"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6153,7 +6153,7 @@
         <v>197</v>
       </c>
       <c r="C183" s="4" t="n">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D183" s="3" t="n">
         <v>280</v>
@@ -6461,7 +6461,7 @@
         <v>213</v>
       </c>
       <c r="C193" s="5" t="n">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="D193" s="3" t="n">
         <v>290</v>
@@ -6769,7 +6769,7 @@
         <v>232</v>
       </c>
       <c r="C203" s="4" t="n">
-        <v>334</v>
+        <v>338</v>
       </c>
       <c r="D203" s="3" t="inlineStr"/>
       <c r="E203" s="3" t="inlineStr">
@@ -6798,7 +6798,7 @@
         <v>233</v>
       </c>
       <c r="C204" s="5" t="n">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="D204" s="3" t="inlineStr"/>
       <c r="E204" s="3" t="inlineStr">
@@ -7167,8 +7167,8 @@
       <c r="B216" s="3" t="n">
         <v>246</v>
       </c>
-      <c r="C216" s="5" t="n">
-        <v>282</v>
+      <c r="C216" s="4" t="n">
+        <v>283</v>
       </c>
       <c r="D216" s="3" t="n">
         <v>294</v>
@@ -7472,7 +7472,7 @@
         <v>258</v>
       </c>
       <c r="C226" s="4" t="n">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="D226" s="3" t="inlineStr"/>
       <c r="E226" s="3" t="inlineStr">
@@ -7501,7 +7501,7 @@
         <v>259</v>
       </c>
       <c r="C227" s="4" t="n">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="D227" s="3" t="inlineStr"/>
       <c r="E227" s="3" t="inlineStr">
@@ -7530,7 +7530,7 @@
         <v>260</v>
       </c>
       <c r="C228" s="5" t="n">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="D228" s="3" t="inlineStr"/>
       <c r="E228" s="3" t="inlineStr">
@@ -7652,7 +7652,7 @@
         <v>265</v>
       </c>
       <c r="C232" s="5" t="n">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D232" s="3" t="n">
         <v>291</v>
@@ -7745,7 +7745,7 @@
         <v>268</v>
       </c>
       <c r="C235" s="4" t="n">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="D235" s="3" t="inlineStr"/>
       <c r="E235" s="3" t="inlineStr">
@@ -7895,8 +7895,8 @@
       <c r="B240" s="3" t="n">
         <v>273</v>
       </c>
-      <c r="C240" s="4" t="n">
-        <v>339</v>
+      <c r="C240" s="5" t="n">
+        <v>307</v>
       </c>
       <c r="D240" s="3" t="inlineStr"/>
       <c r="E240" s="3" t="inlineStr">
@@ -7925,7 +7925,7 @@
         <v>274</v>
       </c>
       <c r="C241" s="5" t="n">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="D241" s="3" t="n">
         <v>293</v>
@@ -8080,7 +8080,7 @@
         <v>280</v>
       </c>
       <c r="C246" s="4" t="n">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="D246" s="3" t="inlineStr"/>
       <c r="E246" s="3" t="inlineStr">
@@ -8109,7 +8109,7 @@
         <v>281</v>
       </c>
       <c r="C247" s="4" t="n">
-        <v>345</v>
+        <v>337</v>
       </c>
       <c r="D247" s="3" t="inlineStr"/>
       <c r="E247" s="3" t="inlineStr">
@@ -8200,7 +8200,7 @@
         <v>284</v>
       </c>
       <c r="C250" s="5" t="n">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D250" s="3" t="n">
         <v>299</v>
@@ -8353,7 +8353,7 @@
         <v>292</v>
       </c>
       <c r="C255" s="5" t="n">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="D255" s="3" t="inlineStr"/>
       <c r="E255" s="3" t="inlineStr">
@@ -8413,7 +8413,7 @@
         <v>294</v>
       </c>
       <c r="C257" s="4" t="n">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="D257" s="3" t="inlineStr"/>
       <c r="E257" s="3" t="inlineStr">
@@ -8442,7 +8442,7 @@
         <v>296</v>
       </c>
       <c r="C258" s="5" t="n">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="D258" s="3" t="inlineStr"/>
       <c r="E258" s="3" t="inlineStr">
@@ -8471,7 +8471,7 @@
         <v>297</v>
       </c>
       <c r="C259" s="5" t="n">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="D259" s="3" t="inlineStr"/>
       <c r="E259" s="3" t="inlineStr">
@@ -8562,7 +8562,7 @@
         <v>300</v>
       </c>
       <c r="C262" s="5" t="n">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="D262" s="3" t="n">
         <v>269</v>
@@ -8593,7 +8593,7 @@
         <v>301</v>
       </c>
       <c r="C263" s="5" t="n">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D263" s="3" t="n">
         <v>300</v>
@@ -8746,7 +8746,7 @@
         <v>309</v>
       </c>
       <c r="C268" s="5" t="n">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="D268" s="3" t="inlineStr"/>
       <c r="E268" s="3" t="inlineStr">
@@ -8775,7 +8775,7 @@
         <v>310</v>
       </c>
       <c r="C269" s="5" t="n">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="D269" s="3" t="inlineStr"/>
       <c r="E269" s="3" t="inlineStr">
@@ -8804,7 +8804,7 @@
         <v>311</v>
       </c>
       <c r="C270" s="5" t="n">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="D270" s="3" t="inlineStr"/>
       <c r="E270" s="3" t="inlineStr">
@@ -8862,7 +8862,7 @@
         <v>314</v>
       </c>
       <c r="C272" s="5" t="n">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="D272" s="3" t="inlineStr"/>
       <c r="E272" s="3" t="inlineStr">
@@ -8922,7 +8922,7 @@
         <v>317</v>
       </c>
       <c r="C274" s="5" t="n">
-        <v>338</v>
+        <v>355</v>
       </c>
       <c r="D274" s="3" t="inlineStr"/>
       <c r="E274" s="3" t="inlineStr">
@@ -8942,146 +8942,146 @@
       </c>
     </row>
     <row r="275">
-      <c r="A275" s="8" t="inlineStr">
+      <c r="A275" s="6" t="inlineStr">
+        <is>
+          <t>RB98</t>
+        </is>
+      </c>
+      <c r="B275" s="3" t="n">
+        <v>321</v>
+      </c>
+      <c r="C275" s="5" t="n">
+        <v>366</v>
+      </c>
+      <c r="D275" s="3" t="inlineStr"/>
+      <c r="E275" s="3" t="inlineStr">
+        <is>
+          <t>Audric Estime</t>
+        </is>
+      </c>
+      <c r="F275" s="3" t="inlineStr">
+        <is>
+          <t>NO (8)</t>
+        </is>
+      </c>
+      <c r="G275" s="3" t="inlineStr">
+        <is>
+          <t>RB</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="8" t="inlineStr">
         <is>
           <t>TE39</t>
         </is>
       </c>
-      <c r="B275" s="3" t="n">
+      <c r="B276" s="3" t="n">
         <v>322</v>
       </c>
-      <c r="C275" s="5" t="n">
+      <c r="C276" s="5" t="n">
         <v>283</v>
       </c>
-      <c r="D275" s="3" t="n">
+      <c r="D276" s="3" t="n">
         <v>282</v>
       </c>
-      <c r="E275" s="3" t="inlineStr">
+      <c r="E276" s="3" t="inlineStr">
         <is>
           <t>Darnell Washington</t>
         </is>
       </c>
-      <c r="F275" s="3" t="inlineStr">
+      <c r="F276" s="3" t="inlineStr">
         <is>
           <t>PIT (9)</t>
         </is>
       </c>
-      <c r="G275" s="3" t="inlineStr">
+      <c r="G276" s="3" t="inlineStr">
         <is>
           <t>TE</t>
         </is>
       </c>
     </row>
-    <row r="276">
-      <c r="A276" s="2" t="inlineStr">
+    <row r="277">
+      <c r="A277" s="2" t="inlineStr">
         <is>
           <t>WR112</t>
         </is>
       </c>
-      <c r="B276" s="3" t="n">
+      <c r="B277" s="3" t="n">
         <v>324</v>
       </c>
-      <c r="C276" s="5" t="n">
-        <v>366</v>
-      </c>
-      <c r="D276" s="3" t="inlineStr"/>
-      <c r="E276" s="3" t="inlineStr">
-        <is>
-          <t>Cedric Tillman</t>
-        </is>
-      </c>
-      <c r="F276" s="3" t="inlineStr">
-        <is>
-          <t>CLE (11)</t>
-        </is>
-      </c>
-      <c r="G276" s="3" t="inlineStr">
-        <is>
-          <t>WR</t>
-        </is>
-      </c>
-    </row>
-    <row r="277">
-      <c r="A277" s="6" t="inlineStr">
-        <is>
-          <t>RB100</t>
-        </is>
-      </c>
-      <c r="B277" s="3" t="n">
-        <v>326</v>
-      </c>
       <c r="C277" s="5" t="n">
-        <v>314</v>
+        <v>372</v>
       </c>
       <c r="D277" s="3" t="inlineStr"/>
       <c r="E277" s="3" t="inlineStr">
         <is>
+          <t>Cedric Tillman</t>
+        </is>
+      </c>
+      <c r="F277" s="3" t="inlineStr">
+        <is>
+          <t>CLE (11)</t>
+        </is>
+      </c>
+      <c r="G277" s="3" t="inlineStr">
+        <is>
+          <t>WR</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="6" t="inlineStr">
+        <is>
+          <t>RB100</t>
+        </is>
+      </c>
+      <c r="B278" s="3" t="n">
+        <v>326</v>
+      </c>
+      <c r="C278" s="5" t="n">
+        <v>314</v>
+      </c>
+      <c r="D278" s="3" t="inlineStr"/>
+      <c r="E278" s="3" t="inlineStr">
+        <is>
           <t>Kareem Hunt</t>
         </is>
       </c>
-      <c r="F277" s="3" t="inlineStr">
+      <c r="F278" s="3" t="inlineStr">
         <is>
           <t>FA ()</t>
         </is>
       </c>
-      <c r="G277" s="3" t="inlineStr">
+      <c r="G278" s="3" t="inlineStr">
         <is>
           <t>RB</t>
-        </is>
-      </c>
-    </row>
-    <row r="278">
-      <c r="A278" s="2" t="inlineStr">
-        <is>
-          <t>WR114</t>
-        </is>
-      </c>
-      <c r="B278" s="3" t="n">
-        <v>328</v>
-      </c>
-      <c r="C278" s="5" t="n">
-        <v>297</v>
-      </c>
-      <c r="D278" s="3" t="n">
-        <v>274</v>
-      </c>
-      <c r="E278" s="3" t="inlineStr">
-        <is>
-          <t>Luke McCaffrey</t>
-        </is>
-      </c>
-      <c r="F278" s="3" t="inlineStr">
-        <is>
-          <t>WAS (7)</t>
-        </is>
-      </c>
-      <c r="G278" s="3" t="inlineStr">
-        <is>
-          <t>WR</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" s="2" t="inlineStr">
         <is>
-          <t>WR115</t>
+          <t>WR114</t>
         </is>
       </c>
       <c r="B279" s="3" t="n">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="C279" s="5" t="n">
-        <v>368</v>
-      </c>
-      <c r="D279" s="3" t="inlineStr"/>
+        <v>297</v>
+      </c>
+      <c r="D279" s="3" t="n">
+        <v>274</v>
+      </c>
       <c r="E279" s="3" t="inlineStr">
         <is>
-          <t>Tez Johnson</t>
+          <t>Luke McCaffrey</t>
         </is>
       </c>
       <c r="F279" s="3" t="inlineStr">
         <is>
-          <t>TB (10)</t>
+          <t>WAS (7)</t>
         </is>
       </c>
       <c r="G279" s="3" t="inlineStr">
@@ -9093,26 +9093,24 @@
     <row r="280">
       <c r="A280" s="2" t="inlineStr">
         <is>
-          <t>WR116</t>
+          <t>WR115</t>
         </is>
       </c>
       <c r="B280" s="3" t="n">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="C280" s="5" t="n">
-        <v>270</v>
-      </c>
-      <c r="D280" s="3" t="n">
-        <v>241</v>
-      </c>
+        <v>369</v>
+      </c>
+      <c r="D280" s="3" t="inlineStr"/>
       <c r="E280" s="3" t="inlineStr">
         <is>
-          <t>Jahan Dotson</t>
+          <t>Tez Johnson</t>
         </is>
       </c>
       <c r="F280" s="3" t="inlineStr">
         <is>
-          <t>ATL (11)</t>
+          <t>TB (10)</t>
         </is>
       </c>
       <c r="G280" s="3" t="inlineStr">
@@ -9124,108 +9122,110 @@
     <row r="281">
       <c r="A281" s="2" t="inlineStr">
         <is>
+          <t>WR116</t>
+        </is>
+      </c>
+      <c r="B281" s="3" t="n">
+        <v>330</v>
+      </c>
+      <c r="C281" s="5" t="n">
+        <v>270</v>
+      </c>
+      <c r="D281" s="3" t="n">
+        <v>241</v>
+      </c>
+      <c r="E281" s="3" t="inlineStr">
+        <is>
+          <t>Jahan Dotson</t>
+        </is>
+      </c>
+      <c r="F281" s="3" t="inlineStr">
+        <is>
+          <t>ATL (11)</t>
+        </is>
+      </c>
+      <c r="G281" s="3" t="inlineStr">
+        <is>
+          <t>WR</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="2" t="inlineStr">
+        <is>
           <t>WR117</t>
         </is>
       </c>
-      <c r="B281" s="3" t="n">
+      <c r="B282" s="3" t="n">
         <v>331</v>
       </c>
-      <c r="C281" s="5" t="n">
+      <c r="C282" s="5" t="n">
         <v>341</v>
-      </c>
-      <c r="D281" s="3" t="inlineStr"/>
-      <c r="E281" s="3" t="inlineStr">
-        <is>
-          <t>Jalen Royals</t>
-        </is>
-      </c>
-      <c r="F281" s="3" t="inlineStr">
-        <is>
-          <t>KC (5)</t>
-        </is>
-      </c>
-      <c r="G281" s="3" t="inlineStr">
-        <is>
-          <t>WR</t>
-        </is>
-      </c>
-    </row>
-    <row r="282">
-      <c r="A282" s="8" t="inlineStr">
-        <is>
-          <t>TE40</t>
-        </is>
-      </c>
-      <c r="B282" s="3" t="n">
-        <v>332</v>
-      </c>
-      <c r="C282" s="5" t="n">
-        <v>378</v>
       </c>
       <c r="D282" s="3" t="inlineStr"/>
       <c r="E282" s="3" t="inlineStr">
         <is>
+          <t>Jalen Royals</t>
+        </is>
+      </c>
+      <c r="F282" s="3" t="inlineStr">
+        <is>
+          <t>KC (5)</t>
+        </is>
+      </c>
+      <c r="G282" s="3" t="inlineStr">
+        <is>
+          <t>WR</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="8" t="inlineStr">
+        <is>
+          <t>TE40</t>
+        </is>
+      </c>
+      <c r="B283" s="3" t="n">
+        <v>332</v>
+      </c>
+      <c r="C283" s="5" t="n">
+        <v>379</v>
+      </c>
+      <c r="D283" s="3" t="inlineStr"/>
+      <c r="E283" s="3" t="inlineStr">
+        <is>
           <t>Max Klare</t>
         </is>
       </c>
-      <c r="F282" s="3" t="inlineStr">
+      <c r="F283" s="3" t="inlineStr">
         <is>
           <t>LAR (11)</t>
         </is>
       </c>
-      <c r="G282" s="3" t="inlineStr">
+      <c r="G283" s="3" t="inlineStr">
         <is>
           <t>TE</t>
-        </is>
-      </c>
-    </row>
-    <row r="283">
-      <c r="A283" s="2" t="inlineStr">
-        <is>
-          <t>WR118</t>
-        </is>
-      </c>
-      <c r="B283" s="3" t="n">
-        <v>333</v>
-      </c>
-      <c r="C283" s="5" t="n">
-        <v>205</v>
-      </c>
-      <c r="D283" s="3" t="n">
-        <v>216</v>
-      </c>
-      <c r="E283" s="3" t="inlineStr">
-        <is>
-          <t>Caleb Douglas</t>
-        </is>
-      </c>
-      <c r="F283" s="3" t="inlineStr">
-        <is>
-          <t>MIA (6)</t>
-        </is>
-      </c>
-      <c r="G283" s="3" t="inlineStr">
-        <is>
-          <t>WR</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" s="2" t="inlineStr">
         <is>
-          <t>WR120</t>
+          <t>WR118</t>
         </is>
       </c>
       <c r="B284" s="3" t="n">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="C284" s="5" t="n">
-        <v>358</v>
-      </c>
-      <c r="D284" s="3" t="inlineStr"/>
+        <v>205</v>
+      </c>
+      <c r="D284" s="3" t="n">
+        <v>216</v>
+      </c>
       <c r="E284" s="3" t="inlineStr">
         <is>
-          <t>Jalen Tolbert</t>
+          <t>Caleb Douglas</t>
         </is>
       </c>
       <c r="F284" s="3" t="inlineStr">
@@ -9242,84 +9242,84 @@
     <row r="285">
       <c r="A285" s="2" t="inlineStr">
         <is>
-          <t>WR122</t>
+          <t>WR120</t>
         </is>
       </c>
       <c r="B285" s="3" t="n">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="C285" s="5" t="n">
-        <v>323</v>
+        <v>358</v>
       </c>
       <c r="D285" s="3" t="inlineStr"/>
       <c r="E285" s="3" t="inlineStr">
         <is>
+          <t>Jalen Tolbert</t>
+        </is>
+      </c>
+      <c r="F285" s="3" t="inlineStr">
+        <is>
+          <t>MIA (6)</t>
+        </is>
+      </c>
+      <c r="G285" s="3" t="inlineStr">
+        <is>
+          <t>WR</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" s="2" t="inlineStr">
+        <is>
+          <t>WR122</t>
+        </is>
+      </c>
+      <c r="B286" s="3" t="n">
+        <v>337</v>
+      </c>
+      <c r="C286" s="5" t="n">
+        <v>324</v>
+      </c>
+      <c r="D286" s="3" t="inlineStr"/>
+      <c r="E286" s="3" t="inlineStr">
+        <is>
           <t>Joshua Palmer</t>
         </is>
       </c>
-      <c r="F285" s="3" t="inlineStr">
+      <c r="F286" s="3" t="inlineStr">
         <is>
           <t>BUF (7)</t>
         </is>
       </c>
-      <c r="G285" s="3" t="inlineStr">
-        <is>
-          <t>WR</t>
-        </is>
-      </c>
-    </row>
-    <row r="286">
-      <c r="A286" s="8" t="inlineStr">
-        <is>
-          <t>TE41</t>
-        </is>
-      </c>
-      <c r="B286" s="3" t="n">
-        <v>338</v>
-      </c>
-      <c r="C286" s="5" t="n">
-        <v>282</v>
-      </c>
-      <c r="D286" s="3" t="n">
-        <v>281</v>
-      </c>
-      <c r="E286" s="3" t="inlineStr">
-        <is>
-          <t>Michael Mayer</t>
-        </is>
-      </c>
-      <c r="F286" s="3" t="inlineStr">
-        <is>
-          <t>LV (13)</t>
-        </is>
-      </c>
       <c r="G286" s="3" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>WR</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" s="8" t="inlineStr">
         <is>
-          <t>TE42</t>
+          <t>TE41</t>
         </is>
       </c>
       <c r="B287" s="3" t="n">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="C287" s="5" t="n">
-        <v>318</v>
-      </c>
-      <c r="D287" s="3" t="inlineStr"/>
+        <v>282</v>
+      </c>
+      <c r="D287" s="3" t="n">
+        <v>281</v>
+      </c>
       <c r="E287" s="3" t="inlineStr">
         <is>
-          <t>Elijah Arroyo</t>
+          <t>Michael Mayer</t>
         </is>
       </c>
       <c r="F287" s="3" t="inlineStr">
         <is>
-          <t>SEA (11)</t>
+          <t>LV (13)</t>
         </is>
       </c>
       <c r="G287" s="3" t="inlineStr">
@@ -9331,24 +9331,24 @@
     <row r="288">
       <c r="A288" s="8" t="inlineStr">
         <is>
-          <t>TE43</t>
+          <t>TE42</t>
         </is>
       </c>
       <c r="B288" s="3" t="n">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="C288" s="5" t="n">
-        <v>373</v>
+        <v>319</v>
       </c>
       <c r="D288" s="3" t="inlineStr"/>
       <c r="E288" s="3" t="inlineStr">
         <is>
-          <t>Tyler Higbee</t>
+          <t>Elijah Arroyo</t>
         </is>
       </c>
       <c r="F288" s="3" t="inlineStr">
         <is>
-          <t>LAR (11)</t>
+          <t>SEA (11)</t>
         </is>
       </c>
       <c r="G288" s="3" t="inlineStr">
@@ -9358,42 +9358,42 @@
       </c>
     </row>
     <row r="289">
-      <c r="A289" s="10" t="inlineStr">
-        <is>
-          <t>QB37</t>
+      <c r="A289" s="8" t="inlineStr">
+        <is>
+          <t>TE43</t>
         </is>
       </c>
       <c r="B289" s="3" t="n">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="C289" s="5" t="n">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="D289" s="3" t="inlineStr"/>
       <c r="E289" s="3" t="inlineStr">
         <is>
-          <t>Mac Jones</t>
+          <t>Tyler Higbee</t>
         </is>
       </c>
       <c r="F289" s="3" t="inlineStr">
         <is>
-          <t>SF (8)</t>
+          <t>LAR (11)</t>
         </is>
       </c>
       <c r="G289" s="3" t="inlineStr">
         <is>
-          <t>QB</t>
+          <t>TE</t>
         </is>
       </c>
     </row>
     <row r="290">
-      <c r="A290" s="8" t="inlineStr">
-        <is>
-          <t>TE45</t>
+      <c r="A290" s="10" t="inlineStr">
+        <is>
+          <t>QB37</t>
         </is>
       </c>
       <c r="B290" s="3" t="n">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="C290" s="5" t="n">
         <v>377</v>
@@ -9401,128 +9401,128 @@
       <c r="D290" s="3" t="inlineStr"/>
       <c r="E290" s="3" t="inlineStr">
         <is>
-          <t>Dawson Knox</t>
+          <t>Mac Jones</t>
         </is>
       </c>
       <c r="F290" s="3" t="inlineStr">
         <is>
-          <t>BUF (7)</t>
+          <t>SF (8)</t>
         </is>
       </c>
       <c r="G290" s="3" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>QB</t>
         </is>
       </c>
     </row>
     <row r="291">
-      <c r="A291" s="10" t="inlineStr">
-        <is>
-          <t>QB38</t>
+      <c r="A291" s="8" t="inlineStr">
+        <is>
+          <t>TE45</t>
         </is>
       </c>
       <c r="B291" s="3" t="n">
-        <v>348</v>
+        <v>344</v>
       </c>
       <c r="C291" s="5" t="n">
-        <v>340</v>
+        <v>378</v>
       </c>
       <c r="D291" s="3" t="inlineStr"/>
       <c r="E291" s="3" t="inlineStr">
         <is>
-          <t>Carson Beck</t>
+          <t>Dawson Knox</t>
         </is>
       </c>
       <c r="F291" s="3" t="inlineStr">
         <is>
-          <t>ARI (14)</t>
+          <t>BUF (7)</t>
         </is>
       </c>
       <c r="G291" s="3" t="inlineStr">
         <is>
-          <t>QB</t>
+          <t>TE</t>
         </is>
       </c>
     </row>
     <row r="292">
-      <c r="A292" s="8" t="inlineStr">
-        <is>
-          <t>TE47</t>
+      <c r="A292" s="10" t="inlineStr">
+        <is>
+          <t>QB38</t>
         </is>
       </c>
       <c r="B292" s="3" t="n">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="C292" s="5" t="n">
-        <v>369</v>
+        <v>340</v>
       </c>
       <c r="D292" s="3" t="inlineStr"/>
       <c r="E292" s="3" t="inlineStr">
         <is>
-          <t>Cole Kmet</t>
+          <t>Carson Beck</t>
         </is>
       </c>
       <c r="F292" s="3" t="inlineStr">
         <is>
-          <t>CHI (10)</t>
+          <t>ARI (14)</t>
         </is>
       </c>
       <c r="G292" s="3" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>QB</t>
         </is>
       </c>
     </row>
     <row r="293">
-      <c r="A293" s="2" t="inlineStr">
-        <is>
-          <t>WR124</t>
+      <c r="A293" s="8" t="inlineStr">
+        <is>
+          <t>TE47</t>
         </is>
       </c>
       <c r="B293" s="3" t="n">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="C293" s="5" t="n">
-        <v>355</v>
+        <v>370</v>
       </c>
       <c r="D293" s="3" t="inlineStr"/>
       <c r="E293" s="3" t="inlineStr">
         <is>
-          <t>Brenen Thompson</t>
+          <t>Cole Kmet</t>
         </is>
       </c>
       <c r="F293" s="3" t="inlineStr">
         <is>
-          <t>LAC (7)</t>
+          <t>CHI (10)</t>
         </is>
       </c>
       <c r="G293" s="3" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>TE</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="A294" s="2" t="inlineStr">
         <is>
-          <t>WR125</t>
+          <t>WR124</t>
         </is>
       </c>
       <c r="B294" s="3" t="n">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="C294" s="5" t="n">
-        <v>299</v>
+        <v>354</v>
       </c>
       <c r="D294" s="3" t="inlineStr"/>
       <c r="E294" s="3" t="inlineStr">
         <is>
-          <t>DeMario Douglas</t>
+          <t>Brenen Thompson</t>
         </is>
       </c>
       <c r="F294" s="3" t="inlineStr">
         <is>
-          <t>NE (11)</t>
+          <t>LAC (7)</t>
         </is>
       </c>
       <c r="G294" s="3" t="inlineStr">
@@ -9534,24 +9534,24 @@
     <row r="295">
       <c r="A295" s="2" t="inlineStr">
         <is>
-          <t>WR126</t>
+          <t>WR125</t>
         </is>
       </c>
       <c r="B295" s="3" t="n">
-        <v>355</v>
+        <v>351</v>
       </c>
       <c r="C295" s="5" t="n">
-        <v>321</v>
+        <v>299</v>
       </c>
       <c r="D295" s="3" t="inlineStr"/>
       <c r="E295" s="3" t="inlineStr">
         <is>
-          <t>Bryce Lance</t>
+          <t>DeMario Douglas</t>
         </is>
       </c>
       <c r="F295" s="3" t="inlineStr">
         <is>
-          <t>NO (8)</t>
+          <t>NE (11)</t>
         </is>
       </c>
       <c r="G295" s="3" t="inlineStr">
@@ -9563,115 +9563,115 @@
     <row r="296">
       <c r="A296" s="2" t="inlineStr">
         <is>
+          <t>WR126</t>
+        </is>
+      </c>
+      <c r="B296" s="3" t="n">
+        <v>355</v>
+      </c>
+      <c r="C296" s="5" t="n">
+        <v>322</v>
+      </c>
+      <c r="D296" s="3" t="inlineStr"/>
+      <c r="E296" s="3" t="inlineStr">
+        <is>
+          <t>Bryce Lance</t>
+        </is>
+      </c>
+      <c r="F296" s="3" t="inlineStr">
+        <is>
+          <t>NO (8)</t>
+        </is>
+      </c>
+      <c r="G296" s="3" t="inlineStr">
+        <is>
+          <t>WR</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" s="2" t="inlineStr">
+        <is>
           <t>WR128</t>
         </is>
       </c>
-      <c r="B296" s="3" t="n">
+      <c r="B297" s="3" t="n">
         <v>358</v>
       </c>
-      <c r="C296" s="5" t="n">
+      <c r="C297" s="5" t="n">
         <v>287</v>
       </c>
-      <c r="D296" s="3" t="n">
+      <c r="D297" s="3" t="n">
         <v>273</v>
       </c>
-      <c r="E296" s="3" t="inlineStr">
+      <c r="E297" s="3" t="inlineStr">
         <is>
           <t>Xavier Hutchinson</t>
         </is>
       </c>
-      <c r="F296" s="3" t="inlineStr">
+      <c r="F297" s="3" t="inlineStr">
         <is>
           <t>HOU (8)</t>
         </is>
       </c>
-      <c r="G296" s="3" t="inlineStr">
-        <is>
-          <t>WR</t>
-        </is>
-      </c>
-    </row>
-    <row r="297">
-      <c r="A297" s="6" t="inlineStr">
+      <c r="G297" s="3" t="inlineStr">
+        <is>
+          <t>WR</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" s="6" t="inlineStr">
         <is>
           <t>RB104</t>
         </is>
       </c>
-      <c r="B297" s="3" t="n">
+      <c r="B298" s="3" t="n">
         <v>360</v>
       </c>
-      <c r="C297" s="5" t="n">
-        <v>350</v>
-      </c>
-      <c r="D297" s="3" t="inlineStr"/>
-      <c r="E297" s="3" t="inlineStr">
+      <c r="C298" s="5" t="n">
+        <v>349</v>
+      </c>
+      <c r="D298" s="3" t="inlineStr"/>
+      <c r="E298" s="3" t="inlineStr">
         <is>
           <t>Jawhar Jordan</t>
         </is>
       </c>
-      <c r="F297" s="3" t="inlineStr">
+      <c r="F298" s="3" t="inlineStr">
         <is>
           <t>HOU (8)</t>
         </is>
       </c>
-      <c r="G297" s="3" t="inlineStr">
+      <c r="G298" s="3" t="inlineStr">
         <is>
           <t>RB</t>
-        </is>
-      </c>
-    </row>
-    <row r="298">
-      <c r="A298" s="2" t="inlineStr">
-        <is>
-          <t>WR130</t>
-        </is>
-      </c>
-      <c r="B298" s="3" t="n">
-        <v>363</v>
-      </c>
-      <c r="C298" s="5" t="n">
-        <v>249</v>
-      </c>
-      <c r="D298" s="3" t="n">
-        <v>229</v>
-      </c>
-      <c r="E298" s="3" t="inlineStr">
-        <is>
-          <t>Treylon Burks</t>
-        </is>
-      </c>
-      <c r="F298" s="3" t="inlineStr">
-        <is>
-          <t>WAS (7)</t>
-        </is>
-      </c>
-      <c r="G298" s="3" t="inlineStr">
-        <is>
-          <t>WR</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="2" t="inlineStr">
         <is>
-          <t>WR132</t>
+          <t>WR130</t>
         </is>
       </c>
       <c r="B299" s="3" t="n">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="C299" s="5" t="n">
-        <v>374</v>
-      </c>
-      <c r="D299" s="3" t="inlineStr"/>
+        <v>249</v>
+      </c>
+      <c r="D299" s="3" t="n">
+        <v>229</v>
+      </c>
       <c r="E299" s="3" t="inlineStr">
         <is>
-          <t>Nick Westbrook-Ikhine</t>
+          <t>Treylon Burks</t>
         </is>
       </c>
       <c r="F299" s="3" t="inlineStr">
         <is>
-          <t>IND (13)</t>
+          <t>WAS (7)</t>
         </is>
       </c>
       <c r="G299" s="3" t="inlineStr">
@@ -9683,24 +9683,24 @@
     <row r="300">
       <c r="A300" s="2" t="inlineStr">
         <is>
-          <t>WR133</t>
+          <t>WR132</t>
         </is>
       </c>
       <c r="B300" s="3" t="n">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="C300" s="5" t="n">
-        <v>359</v>
+        <v>375</v>
       </c>
       <c r="D300" s="3" t="inlineStr"/>
       <c r="E300" s="3" t="inlineStr">
         <is>
-          <t>Savion Williams</t>
+          <t>Nick Westbrook-Ikhine</t>
         </is>
       </c>
       <c r="F300" s="3" t="inlineStr">
         <is>
-          <t>GB (11)</t>
+          <t>IND (13)</t>
         </is>
       </c>
       <c r="G300" s="3" t="inlineStr">
@@ -9710,147 +9710,176 @@
       </c>
     </row>
     <row r="301">
-      <c r="A301" s="6" t="inlineStr">
-        <is>
-          <t>RB107</t>
+      <c r="A301" s="2" t="inlineStr">
+        <is>
+          <t>WR133</t>
         </is>
       </c>
       <c r="B301" s="3" t="n">
-        <v>374</v>
+        <v>367</v>
       </c>
       <c r="C301" s="5" t="n">
-        <v>347</v>
+        <v>359</v>
       </c>
       <c r="D301" s="3" t="inlineStr"/>
       <c r="E301" s="3" t="inlineStr">
         <is>
-          <t>Raheim Sanders</t>
+          <t>Savion Williams</t>
         </is>
       </c>
       <c r="F301" s="3" t="inlineStr">
         <is>
-          <t>CLE (11)</t>
+          <t>GB (11)</t>
         </is>
       </c>
       <c r="G301" s="3" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>WR</t>
         </is>
       </c>
     </row>
     <row r="302">
-      <c r="A302" s="8" t="inlineStr">
-        <is>
-          <t>TE50</t>
+      <c r="A302" s="6" t="inlineStr">
+        <is>
+          <t>RB107</t>
         </is>
       </c>
       <c r="B302" s="3" t="n">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="C302" s="5" t="n">
-        <v>302</v>
+        <v>346</v>
       </c>
       <c r="D302" s="3" t="inlineStr"/>
       <c r="E302" s="3" t="inlineStr">
         <is>
-          <t>Eli Raridon</t>
+          <t>Raheim Sanders</t>
         </is>
       </c>
       <c r="F302" s="3" t="inlineStr">
         <is>
-          <t>NE (11)</t>
+          <t>CLE (11)</t>
         </is>
       </c>
       <c r="G302" s="3" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>RB</t>
         </is>
       </c>
     </row>
     <row r="303">
-      <c r="A303" s="2" t="inlineStr">
-        <is>
-          <t>WR138</t>
+      <c r="A303" s="8" t="inlineStr">
+        <is>
+          <t>TE50</t>
         </is>
       </c>
       <c r="B303" s="3" t="n">
-        <v>383</v>
+        <v>377</v>
       </c>
       <c r="C303" s="5" t="n">
-        <v>360</v>
+        <v>302</v>
       </c>
       <c r="D303" s="3" t="inlineStr"/>
       <c r="E303" s="3" t="inlineStr">
         <is>
-          <t>Zavion Thomas</t>
+          <t>Eli Raridon</t>
         </is>
       </c>
       <c r="F303" s="3" t="inlineStr">
         <is>
-          <t>CHI (10)</t>
+          <t>NE (11)</t>
         </is>
       </c>
       <c r="G303" s="3" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>TE</t>
         </is>
       </c>
     </row>
     <row r="304">
-      <c r="A304" s="6" t="inlineStr">
-        <is>
-          <t>RB109</t>
+      <c r="A304" s="2" t="inlineStr">
+        <is>
+          <t>WR138</t>
         </is>
       </c>
       <c r="B304" s="3" t="n">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="C304" s="5" t="n">
-        <v>352</v>
+        <v>360</v>
       </c>
       <c r="D304" s="3" t="inlineStr"/>
       <c r="E304" s="3" t="inlineStr">
         <is>
+          <t>Zavion Thomas</t>
+        </is>
+      </c>
+      <c r="F304" s="3" t="inlineStr">
+        <is>
+          <t>CHI (10)</t>
+        </is>
+      </c>
+      <c r="G304" s="3" t="inlineStr">
+        <is>
+          <t>WR</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" s="6" t="inlineStr">
+        <is>
+          <t>RB109</t>
+        </is>
+      </c>
+      <c r="B305" s="3" t="n">
+        <v>386</v>
+      </c>
+      <c r="C305" s="5" t="n">
+        <v>351</v>
+      </c>
+      <c r="D305" s="3" t="inlineStr"/>
+      <c r="E305" s="3" t="inlineStr">
+        <is>
           <t>Phil Mafah</t>
         </is>
       </c>
-      <c r="F304" s="3" t="inlineStr">
+      <c r="F305" s="3" t="inlineStr">
         <is>
           <t>DAL (14)</t>
         </is>
       </c>
-      <c r="G304" s="3" t="inlineStr">
+      <c r="G305" s="3" t="inlineStr">
         <is>
           <t>RB</t>
         </is>
       </c>
     </row>
-    <row r="305">
-      <c r="A305" s="8" t="inlineStr">
+    <row r="306">
+      <c r="A306" s="8" t="inlineStr">
         <is>
           <t>TE52</t>
         </is>
       </c>
-      <c r="B305" s="3" t="n">
+      <c r="B306" s="3" t="n">
         <v>387</v>
       </c>
-      <c r="C305" s="5" t="n">
+      <c r="C306" s="5" t="n">
         <v>267</v>
       </c>
-      <c r="D305" s="3" t="n">
+      <c r="D306" s="3" t="n">
         <v>267</v>
       </c>
-      <c r="E305" s="3" t="inlineStr">
+      <c r="E306" s="3" t="inlineStr">
         <is>
           <t>Erick All</t>
         </is>
       </c>
-      <c r="F305" s="3" t="inlineStr">
+      <c r="F306" s="3" t="inlineStr">
         <is>
           <t>CIN (6)</t>
         </is>
       </c>
-      <c r="G305" s="3" t="inlineStr">
+      <c r="G306" s="3" t="inlineStr">
         <is>
           <t>TE</t>
         </is>

</xml_diff>